<commit_message>
updated ankle pads price
</commit_message>
<xml_diff>
--- a/database_ready-latest.xlsx
+++ b/database_ready-latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allan Muli\Desktop\Nexus Frontend project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F49AAE3-CB12-4F49-8466-6AB94FF76196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D60FD0-1AA3-42FD-8DCF-D4228A4DD824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
   </bookViews>
   <sheets>
     <sheet name="database_ready" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="319">
   <si>
     <t>Product_Name</t>
   </si>
@@ -215,9 +215,6 @@
   </si>
   <si>
     <t>Sensory-Proprioception/Gross Motor</t>
-  </si>
-  <si>
-    <t>0.5kgs  3usd/pair,  1kgs 5.7usd/pair , 1.5kgs 9usd/pair  ,2kgs 10.2usd/pair</t>
   </si>
   <si>
     <t>Tear drop hammock</t>
@@ -978,6 +975,15 @@
   </si>
   <si>
     <t>kit</t>
+  </si>
+  <si>
+    <t>2kg pair</t>
+  </si>
+  <si>
+    <t>3kg pair</t>
+  </si>
+  <si>
+    <t>1.5kg pair</t>
   </si>
 </sst>
 </file>
@@ -1821,11 +1827,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33272AF2-EBC5-44E6-A157-58E7ECEB284E}">
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.109375" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
     <col min="3" max="3" width="10.21875" customWidth="1"/>
     <col min="4" max="4" width="73" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" customWidth="1"/>
@@ -1863,7 +1869,7 @@
         <v>1500</v>
       </c>
       <c r="D2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -1883,7 +1889,7 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
@@ -1894,13 +1900,13 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C4">
         <v>500</v>
       </c>
       <c r="D4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F4" t="s">
         <v>12</v>
@@ -1925,7 +1931,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
@@ -1934,7 +1940,7 @@
         <v>4500</v>
       </c>
       <c r="D6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F6" t="s">
         <v>19</v>
@@ -1951,7 +1957,7 @@
         <v>2500</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F7" t="s">
         <v>22</v>
@@ -1993,7 +1999,7 @@
     </row>
     <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -2002,10 +2008,10 @@
         <v>4000</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -2053,7 +2059,7 @@
         <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -2103,7 +2109,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B17" t="s">
         <v>50</v>
@@ -2170,1445 +2176,1482 @@
       <c r="B21" t="s">
         <v>64</v>
       </c>
+      <c r="C21">
+        <v>4500</v>
+      </c>
       <c r="D21" t="s">
-        <v>65</v>
+        <v>316</v>
       </c>
       <c r="F21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C22">
-        <v>12500</v>
+        <v>5000</v>
       </c>
       <c r="D22" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="F22" t="s">
-        <v>68</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C23">
-        <v>7500</v>
+        <v>3500</v>
       </c>
       <c r="D23" t="s">
-        <v>71</v>
+        <v>318</v>
       </c>
       <c r="F23" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="C24">
-        <v>3500</v>
+        <v>12500</v>
       </c>
       <c r="D24" t="s">
-        <v>75</v>
+        <v>297</v>
       </c>
       <c r="F24" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C25">
-        <v>43799</v>
+        <v>7500</v>
       </c>
       <c r="D25" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="F25" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C26">
-        <v>1200</v>
+        <v>3500</v>
+      </c>
+      <c r="D26" t="s">
+        <v>74</v>
       </c>
       <c r="F26" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>282</v>
+        <v>60</v>
       </c>
       <c r="C27">
-        <v>2500</v>
+        <v>43799</v>
+      </c>
+      <c r="D27" t="s">
+        <v>77</v>
       </c>
       <c r="F27" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
-        <v>282</v>
+        <v>80</v>
       </c>
       <c r="C28">
-        <v>3000</v>
+        <v>1200</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C29">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="F29" t="s">
-        <v>272</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>281</v>
       </c>
       <c r="C30">
-        <v>150</v>
+        <v>3000</v>
       </c>
       <c r="F30" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B31" t="s">
-        <v>89</v>
+        <v>282</v>
       </c>
       <c r="C31">
-        <v>500</v>
-      </c>
-      <c r="D31" t="s">
-        <v>92</v>
+        <v>3000</v>
       </c>
       <c r="F31" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C32">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="F32" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B33" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C33">
-        <v>3500</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>294</v>
+        <v>500</v>
+      </c>
+      <c r="D33" t="s">
+        <v>91</v>
       </c>
       <c r="F33" t="s">
-        <v>97</v>
+        <v>272</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34">
+        <v>1000</v>
+      </c>
+      <c r="F34" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B35" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35">
+        <v>3500</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="F35" t="s">
         <v>96</v>
-      </c>
-      <c r="B34" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34">
-        <v>5000</v>
-      </c>
-      <c r="D34" t="s">
-        <v>98</v>
-      </c>
-      <c r="F34" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>99</v>
-      </c>
-      <c r="B35" t="s">
-        <v>279</v>
-      </c>
-      <c r="C35">
-        <v>2000</v>
-      </c>
-      <c r="F35" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="C36">
-        <v>3500</v>
+        <v>5000</v>
+      </c>
+      <c r="D36" t="s">
+        <v>97</v>
       </c>
       <c r="F36" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B37" t="s">
-        <v>35</v>
+        <v>278</v>
       </c>
       <c r="C37">
-        <v>2500</v>
-      </c>
-      <c r="D37" t="s">
-        <v>105</v>
+        <v>2000</v>
       </c>
       <c r="F37" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B38" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C38">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="F38" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B39" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="C39">
-        <v>10000</v>
+        <v>2500</v>
+      </c>
+      <c r="D39" t="s">
+        <v>104</v>
       </c>
       <c r="F39" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B40" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C40">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="F40" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B41" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C41">
-        <v>4000</v>
-      </c>
-      <c r="D41" t="s">
-        <v>299</v>
+        <v>10000</v>
       </c>
       <c r="F41" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="C42">
-        <v>5000</v>
-      </c>
-      <c r="D42" t="s">
-        <v>300</v>
+        <v>10000</v>
       </c>
       <c r="F42" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="B43" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="C43">
-        <v>12500</v>
+        <v>4000</v>
       </c>
       <c r="D43" t="s">
-        <v>16</v>
+        <v>298</v>
       </c>
       <c r="F43" t="s">
-        <v>17</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B44" t="s">
-        <v>280</v>
+        <v>66</v>
       </c>
       <c r="C44">
-        <v>25000</v>
+        <v>5000</v>
+      </c>
+      <c r="D44" t="s">
+        <v>299</v>
       </c>
       <c r="F44" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>120</v>
+        <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>280</v>
+        <v>44</v>
       </c>
       <c r="C45">
-        <v>12000</v>
+        <v>12500</v>
+      </c>
+      <c r="D45" t="s">
+        <v>16</v>
       </c>
       <c r="F45" t="s">
-        <v>121</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>73</v>
+        <v>117</v>
       </c>
       <c r="B46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C46">
-        <v>3500</v>
+        <v>25000</v>
       </c>
       <c r="F46" t="s">
-        <v>76</v>
+        <v>118</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B47" t="s">
-        <v>123</v>
+        <v>279</v>
       </c>
       <c r="C47">
-        <v>4900</v>
+        <v>12000</v>
       </c>
       <c r="F47" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>125</v>
+        <v>72</v>
       </c>
       <c r="B48" t="s">
-        <v>126</v>
+        <v>279</v>
       </c>
       <c r="C48">
-        <v>9000</v>
-      </c>
-      <c r="D48" t="s">
-        <v>127</v>
+        <v>3500</v>
       </c>
       <c r="F48" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B49" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C49">
-        <v>11000</v>
-      </c>
-      <c r="D49" t="s">
-        <v>129</v>
+        <v>4900</v>
       </c>
       <c r="F49" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B50" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="C50">
         <v>9000</v>
       </c>
+      <c r="D50" t="s">
+        <v>126</v>
+      </c>
       <c r="F50" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="B51" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C51">
-        <v>3500</v>
+        <v>11000</v>
+      </c>
+      <c r="D51" t="s">
+        <v>128</v>
       </c>
       <c r="F51" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B52" t="s">
-        <v>136</v>
+        <v>66</v>
       </c>
       <c r="C52">
-        <v>3000</v>
-      </c>
-      <c r="D52" t="s">
-        <v>296</v>
+        <v>9000</v>
       </c>
       <c r="F52" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B53" t="s">
-        <v>67</v>
+        <v>132</v>
       </c>
       <c r="C53">
         <v>3500</v>
       </c>
-      <c r="D53" t="s">
-        <v>139</v>
-      </c>
       <c r="F53" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B54" t="s">
-        <v>67</v>
+        <v>135</v>
       </c>
       <c r="C54">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="D54" t="s">
-        <v>98</v>
+        <v>295</v>
       </c>
       <c r="F54" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>137</v>
+      </c>
+      <c r="B55" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55">
+        <v>3500</v>
+      </c>
+      <c r="D55" t="s">
         <v>138</v>
       </c>
-      <c r="B55" t="s">
-        <v>67</v>
-      </c>
-      <c r="C55">
-        <v>2000</v>
-      </c>
-      <c r="D55" t="s">
-        <v>141</v>
-      </c>
       <c r="F55" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B56" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C56">
-        <v>1200</v>
+        <v>2500</v>
       </c>
       <c r="D56" t="s">
-        <v>142</v>
+        <v>97</v>
       </c>
       <c r="F56" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>312</v>
+        <v>137</v>
       </c>
       <c r="B57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C57">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="D57" t="s">
-        <v>314</v>
+        <v>140</v>
       </c>
       <c r="F57" t="s">
-        <v>313</v>
+        <v>139</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>315</v>
+        <v>137</v>
       </c>
       <c r="B58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C58">
-        <v>15000</v>
+        <v>1200</v>
       </c>
       <c r="D58" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F58" t="s">
-        <v>259</v>
+        <v>139</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="B59" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C59">
-        <v>45000</v>
+        <v>8000</v>
       </c>
       <c r="D59" t="s">
-        <v>144</v>
+        <v>313</v>
       </c>
       <c r="F59" t="s">
-        <v>145</v>
+        <v>312</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>303</v>
+        <v>314</v>
       </c>
       <c r="B60" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C60">
-        <v>55000</v>
+        <v>15000</v>
       </c>
       <c r="D60" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F60" t="s">
-        <v>145</v>
+        <v>258</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B61" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C61">
-        <v>60000</v>
+        <v>45000</v>
       </c>
       <c r="D61" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="F61" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B62" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C62">
-        <v>68000</v>
+        <v>55000</v>
       </c>
       <c r="D62" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>149</v>
+        <v>303</v>
       </c>
       <c r="B63" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="C63">
-        <v>4000</v>
+        <v>60000</v>
       </c>
       <c r="D63" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F63" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>153</v>
+        <v>304</v>
       </c>
       <c r="B64" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C64">
-        <v>3500</v>
+        <v>68000</v>
       </c>
       <c r="D64" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="F64" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="B65" t="s">
-        <v>35</v>
+        <v>149</v>
       </c>
       <c r="C65">
-        <v>200</v>
+        <v>4000</v>
+      </c>
+      <c r="D65" t="s">
+        <v>150</v>
       </c>
       <c r="F65" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B66" t="s">
-        <v>159</v>
+        <v>66</v>
       </c>
       <c r="C66">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="D66" t="s">
-        <v>117</v>
+        <v>153</v>
       </c>
       <c r="F66" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B67" t="s">
-        <v>159</v>
+        <v>35</v>
       </c>
       <c r="C67">
-        <v>1000</v>
-      </c>
-      <c r="D67" t="s">
-        <v>162</v>
+        <v>200</v>
       </c>
       <c r="F67" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B68" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C68">
-        <v>1500</v>
+        <v>500</v>
+      </c>
+      <c r="D68" t="s">
+        <v>116</v>
       </c>
       <c r="F68" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B69" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C69">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="D69" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F69" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="B70" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C70">
-        <v>6000</v>
-      </c>
-      <c r="D70" t="s">
-        <v>36</v>
+        <v>1500</v>
       </c>
       <c r="F70" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="B71" t="s">
-        <v>67</v>
+        <v>167</v>
       </c>
       <c r="C71">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="D71" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="F71" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>291</v>
+        <v>170</v>
       </c>
       <c r="B72" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C72">
-        <v>7500</v>
+        <v>6000</v>
       </c>
       <c r="D72" t="s">
-        <v>290</v>
+        <v>36</v>
       </c>
       <c r="F72" t="s">
-        <v>292</v>
+        <v>172</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B73" t="s">
-        <v>180</v>
+        <v>66</v>
       </c>
       <c r="C73">
-        <v>6000</v>
+        <v>15000</v>
+      </c>
+      <c r="D73" t="s">
+        <v>174</v>
       </c>
       <c r="F73" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>104</v>
+        <v>290</v>
       </c>
       <c r="B74" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="C74">
-        <v>2500</v>
+        <v>7500</v>
       </c>
       <c r="D74" t="s">
-        <v>105</v>
+        <v>289</v>
       </c>
       <c r="F74" t="s">
-        <v>106</v>
+        <v>291</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B75" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C75">
-        <v>45000</v>
-      </c>
-      <c r="D75" t="s">
-        <v>183</v>
+        <v>6000</v>
       </c>
       <c r="F75" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>185</v>
+        <v>103</v>
       </c>
       <c r="B76" t="s">
-        <v>44</v>
+        <v>158</v>
       </c>
       <c r="C76">
-        <v>10000</v>
+        <v>2500</v>
       </c>
       <c r="D76" t="s">
-        <v>186</v>
+        <v>104</v>
       </c>
       <c r="F76" t="s">
-        <v>187</v>
+        <v>105</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B77" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="C77">
-        <v>25000</v>
+        <v>45000</v>
+      </c>
+      <c r="D77" t="s">
+        <v>182</v>
       </c>
       <c r="F77" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B78" t="s">
-        <v>189</v>
+        <v>44</v>
+      </c>
+      <c r="C78">
+        <v>10000</v>
       </c>
       <c r="D78" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="F78" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B79" t="s">
-        <v>10</v>
+        <v>188</v>
+      </c>
+      <c r="C79">
+        <v>25000</v>
       </c>
       <c r="F79" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B80" t="s">
-        <v>10</v>
-      </c>
-      <c r="C80">
-        <v>15000</v>
+        <v>188</v>
+      </c>
+      <c r="D80" t="s">
+        <v>191</v>
       </c>
       <c r="F80" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B81" t="s">
         <v>10</v>
       </c>
-      <c r="C81">
-        <v>2500</v>
-      </c>
       <c r="F81" t="s">
-        <v>274</v>
+        <v>194</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B82" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C82">
         <v>15000</v>
       </c>
-      <c r="D82" t="s">
-        <v>199</v>
-      </c>
       <c r="F82" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B83" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C83">
-        <v>12000</v>
+        <v>2500</v>
       </c>
       <c r="F83" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B84" t="s">
-        <v>159</v>
+        <v>66</v>
       </c>
       <c r="C84">
-        <v>500</v>
+        <v>15000</v>
       </c>
       <c r="D84" t="s">
-        <v>285</v>
+        <v>198</v>
       </c>
       <c r="F84" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B85" t="s">
-        <v>159</v>
+        <v>66</v>
       </c>
       <c r="C85">
-        <v>300</v>
-      </c>
-      <c r="D85" t="s">
-        <v>284</v>
+        <v>12000</v>
       </c>
       <c r="F85" t="s">
-        <v>203</v>
+        <v>274</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B86" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C86">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="D86" t="s">
-        <v>316</v>
+        <v>284</v>
       </c>
       <c r="F86" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B87" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C87">
-        <v>3000</v>
+        <v>300</v>
       </c>
       <c r="D87" t="s">
-        <v>207</v>
+        <v>283</v>
       </c>
       <c r="F87" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B88" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="C88">
-        <v>2000</v>
+        <v>2500</v>
+      </c>
+      <c r="D88" t="s">
+        <v>315</v>
       </c>
       <c r="F88" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B89" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="C89">
-        <v>3500</v>
+        <v>3000</v>
+      </c>
+      <c r="D89" t="s">
+        <v>206</v>
       </c>
       <c r="F89" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B90" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C90">
-        <v>2600</v>
+        <v>2000</v>
       </c>
       <c r="F90" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="B91" t="s">
-        <v>216</v>
+        <v>101</v>
       </c>
       <c r="C91">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="F91" t="s">
-        <v>260</v>
+        <v>211</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>301</v>
+        <v>212</v>
       </c>
       <c r="B92" t="s">
-        <v>218</v>
+        <v>101</v>
       </c>
       <c r="C92">
-        <v>2800</v>
+        <v>2600</v>
       </c>
       <c r="F92" t="s">
-        <v>310</v>
+        <v>213</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>308</v>
+        <v>214</v>
       </c>
       <c r="B93" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C93">
-        <v>3000</v>
-      </c>
-      <c r="D93" t="s">
-        <v>307</v>
+        <v>500</v>
       </c>
       <c r="F93" t="s">
-        <v>309</v>
+        <v>259</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
+        <v>300</v>
+      </c>
+      <c r="B94" t="s">
         <v>217</v>
       </c>
-      <c r="B94" t="s">
-        <v>218</v>
-      </c>
       <c r="C94">
-        <v>3500</v>
-      </c>
-      <c r="D94" t="s">
-        <v>219</v>
+        <v>2800</v>
       </c>
       <c r="F94" t="s">
-        <v>220</v>
+        <v>309</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>221</v>
+        <v>307</v>
       </c>
       <c r="B95" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C95">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="D95" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="F95" t="s">
-        <v>223</v>
+        <v>308</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="B96" t="s">
-        <v>222</v>
+        <v>217</v>
+      </c>
+      <c r="C96">
+        <v>3500</v>
+      </c>
+      <c r="D96" t="s">
+        <v>218</v>
       </c>
       <c r="F96" t="s">
-        <v>276</v>
+        <v>219</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B97" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C97">
-        <v>3000</v>
+        <v>500</v>
+      </c>
+      <c r="D97" t="s">
+        <v>310</v>
       </c>
       <c r="F97" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B98" t="s">
-        <v>281</v>
-      </c>
-      <c r="C98">
-        <v>2800</v>
-      </c>
-      <c r="D98" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="F98" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B99" t="s">
-        <v>168</v>
+        <v>225</v>
       </c>
       <c r="C99">
         <v>3000</v>
       </c>
       <c r="F99" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="B100" t="s">
-        <v>168</v>
+        <v>280</v>
       </c>
       <c r="C100">
-        <v>12500</v>
+        <v>2800</v>
+      </c>
+      <c r="D100" t="s">
+        <v>228</v>
       </c>
       <c r="F100" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B101" t="s">
-        <v>234</v>
+        <v>167</v>
       </c>
       <c r="C101">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="F101" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B102" t="s">
-        <v>234</v>
+        <v>167</v>
       </c>
       <c r="C102">
-        <v>500</v>
+        <v>12500</v>
       </c>
       <c r="F102" t="s">
-        <v>237</v>
+        <v>261</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="B103" t="s">
-        <v>67</v>
+        <v>233</v>
       </c>
       <c r="C103">
-        <v>8500</v>
-      </c>
-      <c r="D103" t="s">
-        <v>239</v>
+        <v>5000</v>
       </c>
       <c r="F103" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B104" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C104">
-        <v>1500</v>
-      </c>
-      <c r="D104" t="s">
-        <v>288</v>
+        <v>500</v>
       </c>
       <c r="F104" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B105" t="s">
-        <v>244</v>
+        <v>66</v>
       </c>
       <c r="C105">
-        <v>2200</v>
+        <v>8500</v>
+      </c>
+      <c r="D105" t="s">
+        <v>238</v>
       </c>
       <c r="F105" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>263</v>
+        <v>240</v>
       </c>
       <c r="B106" t="s">
-        <v>67</v>
+        <v>233</v>
       </c>
       <c r="C106">
-        <v>8500</v>
+        <v>1500</v>
       </c>
       <c r="D106" t="s">
-        <v>246</v>
+        <v>287</v>
       </c>
       <c r="F106" t="s">
-        <v>266</v>
+        <v>241</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="B107" t="s">
-        <v>102</v>
+        <v>243</v>
       </c>
       <c r="C107">
-        <v>2500</v>
+        <v>2200</v>
       </c>
       <c r="F107" t="s">
-        <v>267</v>
+        <v>244</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
+        <v>262</v>
+      </c>
+      <c r="B108" t="s">
+        <v>66</v>
+      </c>
+      <c r="C108">
+        <v>8500</v>
+      </c>
+      <c r="D108" t="s">
+        <v>245</v>
+      </c>
+      <c r="F108" t="s">
         <v>265</v>
-      </c>
-      <c r="B108" t="s">
-        <v>102</v>
-      </c>
-      <c r="C108">
-        <v>1500</v>
-      </c>
-      <c r="F108" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="B109" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C109">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="F109" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="B110" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C110">
         <v>1500</v>
       </c>
       <c r="F110" t="s">
-        <v>250</v>
+        <v>267</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B111" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C111">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F111" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B112" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C112">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="F112" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B113" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C113">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="F113" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B114" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="C114">
+        <v>3000</v>
       </c>
       <c r="F114" t="s">
-        <v>269</v>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>254</v>
+      </c>
+      <c r="B115" t="s">
+        <v>101</v>
+      </c>
+      <c r="C115">
+        <v>3000</v>
+      </c>
+      <c r="F115" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>256</v>
+      </c>
+      <c r="B116" t="s">
+        <v>101</v>
+      </c>
+      <c r="F116" t="s">
+        <v>268</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated the product database with images and price
</commit_message>
<xml_diff>
--- a/database_ready-latest.xlsx
+++ b/database_ready-latest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allan Muli\Desktop\Nexus Frontend project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D60FD0-1AA3-42FD-8DCF-D4228A4DD824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1930222E-EEFF-493A-9492-A2530C8F52F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="575">
   <si>
     <t>Product_Name</t>
   </si>
@@ -984,6 +984,815 @@
   </si>
   <si>
     <t>1.5kg pair</t>
+  </si>
+  <si>
+    <t>Buckle ring game</t>
+  </si>
+  <si>
+    <t>buckle-ring-game.jpg</t>
+  </si>
+  <si>
+    <t>Good builder and developer of kids skills in 
+Sequencing, 
+color identification,
+Fine motor skills
+Cognitive function 
+Matching</t>
+  </si>
+  <si>
+    <t>Fine motor pins</t>
+  </si>
+  <si>
+    <t>fine-motor-pins.jpg</t>
+  </si>
+  <si>
+    <t>Develop fine motor skills as baby learns
+Color sorting, stacking, balance  eye hand coordination</t>
+  </si>
+  <si>
+    <t>Small Portable umbrella</t>
+  </si>
+  <si>
+    <t>small-umbrella.jpg</t>
+  </si>
+  <si>
+    <t>Magnetic Matching Ring Battle</t>
+  </si>
+  <si>
+    <t>Colour identification
+Sorting
+Fine motor
+Cognitive skills development</t>
+  </si>
+  <si>
+    <t>magnetic-ring-game.jpg</t>
+  </si>
+  <si>
+    <t>Rainbow slug fidget</t>
+  </si>
+  <si>
+    <t>For unsettled kids with ADHD and hyperactivity</t>
+  </si>
+  <si>
+    <t>rainbow-slug-fidget.jpg</t>
+  </si>
+  <si>
+    <t>Chart - press for audio</t>
+  </si>
+  <si>
+    <t>Wall chart with audio buttons for voice 
+Perfect support speech practice</t>
+  </si>
+  <si>
+    <t>chart-with-audio.jpg</t>
+  </si>
+  <si>
+    <t>Resistance band</t>
+  </si>
+  <si>
+    <t>resistance-band.jpg</t>
+  </si>
+  <si>
+    <t>3D puzzles STEM</t>
+  </si>
+  <si>
+    <t>The best way to bring Board paper cutouts and construct prices into 3d items</t>
+  </si>
+  <si>
+    <t>3d-puzzles.jpg</t>
+  </si>
+  <si>
+    <t>LED board -  fine motor support</t>
+  </si>
+  <si>
+    <t>Supprt fine motor skills through switch on / off 
+Turn key
+Rotate switch 
+Plug in</t>
+  </si>
+  <si>
+    <t>led-board.jpg</t>
+  </si>
+  <si>
+    <t>Busy Suit ADL Board</t>
+  </si>
+  <si>
+    <t>busy-suit-board.jpg</t>
+  </si>
+  <si>
+    <t>sensory-fidget-band.jpg</t>
+  </si>
+  <si>
+    <t>Sensory &amp; anxiety fidget band</t>
+  </si>
+  <si>
+    <t>No better companion to squash, pull and fidget with in private</t>
+  </si>
+  <si>
+    <t>Audio flash cards</t>
+  </si>
+  <si>
+    <t>With a set of over 90 flash card including:
+Activities
+Alphabets
+Vegetables
+Animals 
+People</t>
+  </si>
+  <si>
+    <t>audio-flash-card.jpg</t>
+  </si>
+  <si>
+    <t>flat-cap.jpg</t>
+  </si>
+  <si>
+    <t>Flat cap</t>
+  </si>
+  <si>
+    <t>Geometric sorter with xylophone &amp; fishing rod</t>
+  </si>
+  <si>
+    <t>geometric-sorter.jpg</t>
+  </si>
+  <si>
+    <t>Bubble gun 2 in 1</t>
+  </si>
+  <si>
+    <t>bubble-gun-2in1.jpg</t>
+  </si>
+  <si>
+    <t>Hand grip Strengthening</t>
+  </si>
+  <si>
+    <t>hand-grip-strengthening.jpg</t>
+  </si>
+  <si>
+    <t>Bubble gun 106</t>
+  </si>
+  <si>
+    <t>bubble-gun-106.jpg</t>
+  </si>
+  <si>
+    <t>Water gel beads</t>
+  </si>
+  <si>
+    <t>Sensory integration balls with water soft feel</t>
+  </si>
+  <si>
+    <t>water-gel-beads.jpg</t>
+  </si>
+  <si>
+    <t>Half foot massage balls</t>
+  </si>
+  <si>
+    <t>half-foot-massage-balls.jpg</t>
+  </si>
+  <si>
+    <t>My first assorted books</t>
+  </si>
+  <si>
+    <t>Great for teaching basic first words pictographic a5 size book</t>
+  </si>
+  <si>
+    <t>assorted-book.jpg</t>
+  </si>
+  <si>
+    <t>Stacking cups 1 player (beginner)</t>
+  </si>
+  <si>
+    <t>With guided pattern let your child improve cognitive, fine motor, eye hand coordination, matching and colour recognition</t>
+  </si>
+  <si>
+    <t>stacking-cups.jpg</t>
+  </si>
+  <si>
+    <t>Fidget Vent ball - Netted big</t>
+  </si>
+  <si>
+    <t>Soft Fidget balls with encouraging action reactions pop out through net</t>
+  </si>
+  <si>
+    <t>fidget-vent-ball.jpg</t>
+  </si>
+  <si>
+    <t>stacking-game.jpg</t>
+  </si>
+  <si>
+    <t>Stacking game</t>
+  </si>
+  <si>
+    <t>Gel crayons 24pcs</t>
+  </si>
+  <si>
+    <t>Bright 
+Washable 
+Twist to expose (no need for sharpening)</t>
+  </si>
+  <si>
+    <t>gel-crayon(24).jpg</t>
+  </si>
+  <si>
+    <t>Sunk magic bk - pre school B5</t>
+  </si>
+  <si>
+    <t>Drawing 
+Alphabet 
+Numbers
+Math</t>
+  </si>
+  <si>
+    <t>sunk-magic-book.jpg</t>
+  </si>
+  <si>
+    <t>1x1m Safety floor Matt - 12mm thick</t>
+  </si>
+  <si>
+    <t>Ensure you therapy play space and kids corner is safeguarded through safety padded mats</t>
+  </si>
+  <si>
+    <t>safety-floor-mat.jpg</t>
+  </si>
+  <si>
+    <t>Sorter fidget ball</t>
+  </si>
+  <si>
+    <t>Finger trainer that help with cognitive colour identification and matching</t>
+  </si>
+  <si>
+    <t>fidget-ball.jpg</t>
+  </si>
+  <si>
+    <t>Pitballs</t>
+  </si>
+  <si>
+    <t>50 pcs plastic pack of medium
+Size multi color strong pot balls</t>
+  </si>
+  <si>
+    <t>pitballs.jpg</t>
+  </si>
+  <si>
+    <t>Fidget spin ball</t>
+  </si>
+  <si>
+    <t>To help ADHDers and those with anxiety to fidget and focus</t>
+  </si>
+  <si>
+    <t>fidget-spin-ball.jpg</t>
+  </si>
+  <si>
+    <t>Sensory brush - glove</t>
+  </si>
+  <si>
+    <t>sensory-brush.jpg</t>
+  </si>
+  <si>
+    <t>Slime with Rubiks Cube</t>
+  </si>
+  <si>
+    <t>slime-with-rubiks.jpg</t>
+  </si>
+  <si>
+    <t>Letters 🧩 puzzle with grip (wooden)</t>
+  </si>
+  <si>
+    <t>letters-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Assorted charts</t>
+  </si>
+  <si>
+    <t>assorted-charts.jpg</t>
+  </si>
+  <si>
+    <t>For the children who you need to keep focused 
+Desk charts are the best support this set is full 12 different pieces</t>
+  </si>
+  <si>
+    <t>Squirrel number puzzle</t>
+  </si>
+  <si>
+    <t>squirrel-number-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Chart B4 scan &amp; listen - 12pcs assorted</t>
+  </si>
+  <si>
+    <t>Speech development for audio visual learners</t>
+  </si>
+  <si>
+    <t>chart-b4-scan.jpg</t>
+  </si>
+  <si>
+    <t>InclusivWear Bucket Hat</t>
+  </si>
+  <si>
+    <t>Inclusive-wear-bucketHat.jpg</t>
+  </si>
+  <si>
+    <t>Pom Pom pack</t>
+  </si>
+  <si>
+    <t>Best for engaging DIY sorting activities</t>
+  </si>
+  <si>
+    <t>pompom-pack.jpg</t>
+  </si>
+  <si>
+    <t>heavy-rebound-ball.jpg</t>
+  </si>
+  <si>
+    <t>Heavy rebound ball</t>
+  </si>
+  <si>
+    <t>Fruits shape sorter</t>
+  </si>
+  <si>
+    <t>2 in one fine motor trainer for child to identify cut and sort the shapes</t>
+  </si>
+  <si>
+    <t>fruit-shape-sorter.jpg</t>
+  </si>
+  <si>
+    <t>Enhance creativity, improve finger movement and fine motor development</t>
+  </si>
+  <si>
+    <t>modelling-clay.jpg</t>
+  </si>
+  <si>
+    <t>Modeling clay</t>
+  </si>
+  <si>
+    <t>3D two head massager</t>
+  </si>
+  <si>
+    <t>Recommend this one for oral
+Muscular face massage to support with speech development, swallowing, drooling</t>
+  </si>
+  <si>
+    <t>3d-head-massager.jpg</t>
+  </si>
+  <si>
+    <t>Places matching puzzle</t>
+  </si>
+  <si>
+    <t>Fine motor skills development
+Eye hand coordination 
+Cognitive skills</t>
+  </si>
+  <si>
+    <t>places-matching-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Shank Magic pen control set</t>
+  </si>
+  <si>
+    <t>Train your baby on how to write and draw with our shaken magic books which comes with pen &amp; grip trainer complete with pen refills</t>
+  </si>
+  <si>
+    <t>magic-pen-controlSet.jpg</t>
+  </si>
+  <si>
+    <t>Fidget ball</t>
+  </si>
+  <si>
+    <t>fidget-ball-large.jpg</t>
+  </si>
+  <si>
+    <t>Fishing rod - level 2</t>
+  </si>
+  <si>
+    <t>Three in one level 2 daiyoutai for fine motor skills, eye hand coordination</t>
+  </si>
+  <si>
+    <t>fishing-rod.jpg</t>
+  </si>
+  <si>
+    <t>Cordless skipping rope</t>
+  </si>
+  <si>
+    <t>Safely Train in vestibular and body movements with your child before graduating to beaded skipping rope</t>
+  </si>
+  <si>
+    <t>cordless-skipping-rope.jpg</t>
+  </si>
+  <si>
+    <t>Teeny Baby Audio story books</t>
+  </si>
+  <si>
+    <t>Short beginner stories for your child with scannable QR code for audio version.
+Teach diction articulation and perfect for audiovisual learners</t>
+  </si>
+  <si>
+    <t>baby-audio-book.jpg</t>
+  </si>
+  <si>
+    <t>Beaded skipping rope</t>
+  </si>
+  <si>
+    <t>With beads adding weight to support beginner skippers</t>
+  </si>
+  <si>
+    <t>beaded-skipping-rope.jpg</t>
+  </si>
+  <si>
+    <t>Cloth sensory chewie</t>
+  </si>
+  <si>
+    <t>High absorption material best  doe kids who drool to avoid wet neckline &amp; colds</t>
+  </si>
+  <si>
+    <t>cloth-chewie.jpg</t>
+  </si>
+  <si>
+    <t>Dough roller</t>
+  </si>
+  <si>
+    <t>Massage roller perfect for those needing sensory integration</t>
+  </si>
+  <si>
+    <t>dough-roller.jpg</t>
+  </si>
+  <si>
+    <t>Dinosaur balance stack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor skills 
+Eye hand coordination </t>
+  </si>
+  <si>
+    <t>dinosaur-balance-stack.jpg</t>
+  </si>
+  <si>
+    <t>Number Maze</t>
+  </si>
+  <si>
+    <t>number-maze.jpg</t>
+  </si>
+  <si>
+    <t>Bingo Ability Game - pocket size</t>
+  </si>
+  <si>
+    <t>bingo-game.jpg</t>
+  </si>
+  <si>
+    <t>Diaoyutai Fine Motor Fish Game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improve concentration, eye hand coordination, patience and fine motor skills and precision </t>
+  </si>
+  <si>
+    <t>diaoyutai-fish-game.jpg</t>
+  </si>
+  <si>
+    <t>2 in 1 rubric vibes - magic cube</t>
+  </si>
+  <si>
+    <t>2in1-rubiks.jpg</t>
+  </si>
+  <si>
+    <t>Balance Chair</t>
+  </si>
+  <si>
+    <t>balance-chair.jpg</t>
+  </si>
+  <si>
+    <t>animal-chart.jpg</t>
+  </si>
+  <si>
+    <t>Charts Animal world A3</t>
+  </si>
+  <si>
+    <t>A dozen set of assorted animals chart to support in speech and recognition 
+Cognitive development of environmental learning</t>
+  </si>
+  <si>
+    <t>Stacking cups 2player</t>
+  </si>
+  <si>
+    <t>speed, colour sorting, eye hand coordination, motor skills</t>
+  </si>
+  <si>
+    <t>stacking-cups-2player.jpg</t>
+  </si>
+  <si>
+    <t>Flash cards set - Card Bus</t>
+  </si>
+  <si>
+    <t>Ride the bus of early learning with our 4 in 1 multiple sets of flash cards</t>
+  </si>
+  <si>
+    <t>card-bus.jpg</t>
+  </si>
+  <si>
+    <t>Slime</t>
+  </si>
+  <si>
+    <t>Large bottle</t>
+  </si>
+  <si>
+    <t>slime-largeBottle.jpg</t>
+  </si>
+  <si>
+    <t>Animal matching puzzle</t>
+  </si>
+  <si>
+    <t>In support of eye had coordination
+Fine motor skills
+Cognitive development</t>
+  </si>
+  <si>
+    <t>animal-matching-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Mini toys - super Mario</t>
+  </si>
+  <si>
+    <t>supermario-toy.jpg</t>
+  </si>
+  <si>
+    <t>Fairy tale books with audio</t>
+  </si>
+  <si>
+    <t>Fairytale fairy 🧚‍♀️ stories for your child with scannable QR code for audio version.</t>
+  </si>
+  <si>
+    <t>fairy-tale-book.jpg</t>
+  </si>
+  <si>
+    <t>Activity timer</t>
+  </si>
+  <si>
+    <t>A child’s teacher for start and stop in activity transition with a ringer ..</t>
+  </si>
+  <si>
+    <t>activity-timer.jpg</t>
+  </si>
+  <si>
+    <t>Magic shaken books set a5</t>
+  </si>
+  <si>
+    <t>Sank magic books are perfect for practicing how to write ✍️</t>
+  </si>
+  <si>
+    <t>magic-shaken-book.jpg</t>
+  </si>
+  <si>
+    <t>Triangle color puzzle</t>
+  </si>
+  <si>
+    <t>For brain gym, teach sizes.
+Improve fine motor development, eye hand coordination and to improve attention</t>
+  </si>
+  <si>
+    <t>triangle-color-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Shadow matched images</t>
+  </si>
+  <si>
+    <t>Help with recognition and build cognitive skills through this brain game</t>
+  </si>
+  <si>
+    <t>shadow-matched-images.jpg</t>
+  </si>
+  <si>
+    <t>Hoodies - Move4Autism</t>
+  </si>
+  <si>
+    <t>hoodies-move4autism.jpg</t>
+  </si>
+  <si>
+    <t>connect-four.jpg</t>
+  </si>
+  <si>
+    <t>Connect four</t>
+  </si>
+  <si>
+    <t>Eye hand coordination
+ Rain trainer for critics thinking</t>
+  </si>
+  <si>
+    <t>Match it - time puzzle</t>
+  </si>
+  <si>
+    <t>Telling time in analog and digital format</t>
+  </si>
+  <si>
+    <t>match-it-game.jpg</t>
+  </si>
+  <si>
+    <t>Grooved grip pencil</t>
+  </si>
+  <si>
+    <t>Training your child to hold a pencil and for handwriting improvement</t>
+  </si>
+  <si>
+    <t>grooved-grip-pencil.jpg</t>
+  </si>
+  <si>
+    <t>Number &amp; Shapes 🧩 puzzle (1-10 with grip)</t>
+  </si>
+  <si>
+    <t>Helps with 
+- Learning shapes
+- Number identification</t>
+  </si>
+  <si>
+    <t>number-and-shapes.jpg</t>
+  </si>
+  <si>
+    <t>Magnetic sticks 25pc</t>
+  </si>
+  <si>
+    <t>Free play and brain gym for kids cognitive n imagination 
+Build the creative &amp; STEM mind</t>
+  </si>
+  <si>
+    <t>magnetic-sticks-25pc.jpg</t>
+  </si>
+  <si>
+    <t>Sun visor</t>
+  </si>
+  <si>
+    <t>sun-visor.jpg</t>
+  </si>
+  <si>
+    <t>Percussion Platform</t>
+  </si>
+  <si>
+    <t>percussion-platform.jpg</t>
+  </si>
+  <si>
+    <t>Hexagonal Prism Cube</t>
+  </si>
+  <si>
+    <t>hexagonal-prism-cube.jpg</t>
+  </si>
+  <si>
+    <t>water-bottle.jpg</t>
+  </si>
+  <si>
+    <t>Water Bottle</t>
+  </si>
+  <si>
+    <t>Hoops</t>
+  </si>
+  <si>
+    <t>For body coordination with gross motor focus</t>
+  </si>
+  <si>
+    <t>hoops.jpg</t>
+  </si>
+  <si>
+    <t>Alarm Clock Shaped Beads</t>
+  </si>
+  <si>
+    <t>alarm-clock-shaped-beads.jpg</t>
+  </si>
+  <si>
+    <t>Vegetable pinch puzzle</t>
+  </si>
+  <si>
+    <t>Help with gripping, fine motor skill, eye hand coordination, identification and teaching gadget for vegetables,</t>
+  </si>
+  <si>
+    <t>vegetable-pinch-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Opposites puzzle</t>
+  </si>
+  <si>
+    <t>Improve cognitive learning of opposites while working on fine motor skills, eye hand coordination</t>
+  </si>
+  <si>
+    <t>Hand Face 3dmassager</t>
+  </si>
+  <si>
+    <t>For muscle relaxation in supper of speech development and drilling control</t>
+  </si>
+  <si>
+    <t>hand-face-3d-facemassager.jpg</t>
+  </si>
+  <si>
+    <t>Wipe clean work books</t>
+  </si>
+  <si>
+    <t>wipe-clean-work-books.jpg</t>
+  </si>
+  <si>
+    <t>Power ball</t>
+  </si>
+  <si>
+    <t>Perfect soft ball for hand &amp; finger muscles exercises</t>
+  </si>
+  <si>
+    <t>power-ball.jpg</t>
+  </si>
+  <si>
+    <t>Short tales with teachings audio picture books</t>
+  </si>
+  <si>
+    <t>Stories for your child with scannable QR code for audio version.</t>
+  </si>
+  <si>
+    <t>short-tales-with-audio.jpg</t>
+  </si>
+  <si>
+    <t>Mochabo &amp; Neuro pals: Inclusive social stories</t>
+  </si>
+  <si>
+    <t>Available multiple formats for all kids despite their level of ability 
+Hard cover - 500/-
+Audiovisual book in flash with sign language- 1800</t>
+  </si>
+  <si>
+    <t>mochabo-and-neuro-pals.jpg</t>
+  </si>
+  <si>
+    <t>2 in 1 Dinosaur magnetic fishing puzzles</t>
+  </si>
+  <si>
+    <t>To improve concentration, fine motor skills, and eye hand coordination plus matching skills</t>
+  </si>
+  <si>
+    <t>2in1-dinosaur-magnetic-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>Pop it children’s hand bag</t>
+  </si>
+  <si>
+    <t>A baby gurls purse with calming activity that you can travel with around and carry on a hanky, toy or any other item you need. 
+Comes complete with the strap</t>
+  </si>
+  <si>
+    <t>pop-it.jpg</t>
+  </si>
+  <si>
+    <t>Numbers with grip 1-20</t>
+  </si>
+  <si>
+    <t>Helps with - Learning shapes,  Number identification, Slot identification &amp; matching,  Fine motor skills development and Eye hands coordination</t>
+  </si>
+  <si>
+    <t>number-with-grip.jpg</t>
+  </si>
+  <si>
+    <t>Wooden puzzles</t>
+  </si>
+  <si>
+    <t>For brain gym, fine motor development, eye hand coordination and to improve attention</t>
+  </si>
+  <si>
+    <t>wooden-puzzles.jpg</t>
+  </si>
+  <si>
+    <t>4D massager</t>
+  </si>
+  <si>
+    <t>Face, hand massager</t>
+  </si>
+  <si>
+    <t>4d-massager.jpg</t>
+  </si>
+  <si>
+    <t>Pen control level 1 A4</t>
+  </si>
+  <si>
+    <t>Train your baby on how to make basic shapes, strokes, train and draw with our sanken magic books which comes with pen &amp; grip trainer complete with pen refills</t>
+  </si>
+  <si>
+    <t>pen-control-level-1.jpg</t>
+  </si>
+  <si>
+    <t>First pocket flash books</t>
+  </si>
+  <si>
+    <t>Convenient pocket book that you can more with and keep practicing to positively engage your child</t>
+  </si>
+  <si>
+    <t>first-pocket-flash-book.jpg</t>
+  </si>
+  <si>
+    <t>Big umbrella</t>
+  </si>
+  <si>
+    <t>big-umbrella.jpg</t>
+  </si>
+  <si>
+    <t>Writing ✍️ set</t>
+  </si>
+  <si>
+    <t>Complete beginner set of grooved pencil rubber and sharpener</t>
+  </si>
+  <si>
+    <t>writing-set.jpg</t>
+  </si>
+  <si>
+    <t>safety</t>
+  </si>
+  <si>
+    <t>opposites-puzzle.jpg</t>
   </si>
 </sst>
 </file>
@@ -1827,15 +2636,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33272AF2-EBC5-44E6-A157-58E7ECEB284E}">
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F211"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.109375" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="1" max="1" width="39.109375" customWidth="1"/>
+    <col min="2" max="2" width="60.6640625" customWidth="1"/>
     <col min="3" max="3" width="10.21875" customWidth="1"/>
-    <col min="4" max="4" width="73" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="30.21875" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="35.44140625" customWidth="1"/>
+    <col min="6" max="6" width="33.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1997,7 +2806,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>285</v>
       </c>
@@ -2007,7 +2816,7 @@
       <c r="C10">
         <v>4000</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>294</v>
       </c>
       <c r="F10" t="s">
@@ -2389,7 +3198,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>95</v>
       </c>
@@ -2399,7 +3208,7 @@
       <c r="C35">
         <v>3500</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" t="s">
         <v>293</v>
       </c>
       <c r="F35" t="s">
@@ -3652,6 +4461,1531 @@
       </c>
       <c r="F116" t="s">
         <v>268</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>319</v>
+      </c>
+      <c r="B117" t="s">
+        <v>101</v>
+      </c>
+      <c r="C117">
+        <v>1600</v>
+      </c>
+      <c r="E117" t="s">
+        <v>321</v>
+      </c>
+      <c r="F117" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>322</v>
+      </c>
+      <c r="B118" t="s">
+        <v>101</v>
+      </c>
+      <c r="C118">
+        <v>3000</v>
+      </c>
+      <c r="D118" t="s">
+        <v>324</v>
+      </c>
+      <c r="F118" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>325</v>
+      </c>
+      <c r="B119" t="s">
+        <v>573</v>
+      </c>
+      <c r="C119">
+        <v>2000</v>
+      </c>
+      <c r="D119" t="s">
+        <v>325</v>
+      </c>
+      <c r="F119" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>327</v>
+      </c>
+      <c r="B120" t="s">
+        <v>101</v>
+      </c>
+      <c r="C120">
+        <v>2000</v>
+      </c>
+      <c r="D120" t="s">
+        <v>328</v>
+      </c>
+      <c r="F120" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>330</v>
+      </c>
+      <c r="B121" t="s">
+        <v>158</v>
+      </c>
+      <c r="C121">
+        <v>1000</v>
+      </c>
+      <c r="D121" t="s">
+        <v>331</v>
+      </c>
+      <c r="F121" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>333</v>
+      </c>
+      <c r="B122" t="s">
+        <v>101</v>
+      </c>
+      <c r="C122">
+        <v>1100</v>
+      </c>
+      <c r="D122" t="s">
+        <v>334</v>
+      </c>
+      <c r="F122" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>336</v>
+      </c>
+      <c r="B123" t="s">
+        <v>60</v>
+      </c>
+      <c r="C123">
+        <v>500</v>
+      </c>
+      <c r="F123" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>338</v>
+      </c>
+      <c r="B124" t="s">
+        <v>101</v>
+      </c>
+      <c r="C124">
+        <v>1500</v>
+      </c>
+      <c r="D124" t="s">
+        <v>339</v>
+      </c>
+      <c r="F124" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>341</v>
+      </c>
+      <c r="B125" t="s">
+        <v>101</v>
+      </c>
+      <c r="C125">
+        <v>2000</v>
+      </c>
+      <c r="D125" t="s">
+        <v>342</v>
+      </c>
+      <c r="F125" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>344</v>
+      </c>
+      <c r="B126" t="s">
+        <v>101</v>
+      </c>
+      <c r="C126">
+        <v>2000</v>
+      </c>
+      <c r="F126" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>347</v>
+      </c>
+      <c r="B127" t="s">
+        <v>158</v>
+      </c>
+      <c r="C127">
+        <v>200</v>
+      </c>
+      <c r="D127" t="s">
+        <v>348</v>
+      </c>
+      <c r="F127" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>349</v>
+      </c>
+      <c r="B128" t="s">
+        <v>221</v>
+      </c>
+      <c r="C128">
+        <v>2000</v>
+      </c>
+      <c r="D128" t="s">
+        <v>350</v>
+      </c>
+      <c r="F128" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>353</v>
+      </c>
+      <c r="B129" t="s">
+        <v>573</v>
+      </c>
+      <c r="C129">
+        <v>1000</v>
+      </c>
+      <c r="F129" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>354</v>
+      </c>
+      <c r="B130" t="s">
+        <v>233</v>
+      </c>
+      <c r="C130">
+        <v>2300</v>
+      </c>
+      <c r="F130" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>356</v>
+      </c>
+      <c r="B131" t="s">
+        <v>233</v>
+      </c>
+      <c r="C131">
+        <v>1200</v>
+      </c>
+      <c r="F131" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>358</v>
+      </c>
+      <c r="B132" t="s">
+        <v>281</v>
+      </c>
+      <c r="C132">
+        <v>600</v>
+      </c>
+      <c r="F132" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>360</v>
+      </c>
+      <c r="B133" t="s">
+        <v>233</v>
+      </c>
+      <c r="C133">
+        <v>1600</v>
+      </c>
+      <c r="F133" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>362</v>
+      </c>
+      <c r="B134" t="s">
+        <v>44</v>
+      </c>
+      <c r="C134">
+        <v>250</v>
+      </c>
+      <c r="D134" t="s">
+        <v>363</v>
+      </c>
+      <c r="F134" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>365</v>
+      </c>
+      <c r="B135" t="s">
+        <v>10</v>
+      </c>
+      <c r="C135">
+        <v>1500</v>
+      </c>
+      <c r="F135" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>367</v>
+      </c>
+      <c r="B136" t="s">
+        <v>101</v>
+      </c>
+      <c r="C136">
+        <v>110</v>
+      </c>
+      <c r="D136" t="s">
+        <v>368</v>
+      </c>
+      <c r="F136" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>370</v>
+      </c>
+      <c r="B137" t="s">
+        <v>233</v>
+      </c>
+      <c r="C137">
+        <v>1500</v>
+      </c>
+      <c r="D137" t="s">
+        <v>371</v>
+      </c>
+      <c r="F137" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>373</v>
+      </c>
+      <c r="B138" t="s">
+        <v>158</v>
+      </c>
+      <c r="C138">
+        <v>600</v>
+      </c>
+      <c r="D138" t="s">
+        <v>374</v>
+      </c>
+      <c r="F138" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>377</v>
+      </c>
+      <c r="B139" t="s">
+        <v>233</v>
+      </c>
+      <c r="C139">
+        <v>2000</v>
+      </c>
+      <c r="F139" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>378</v>
+      </c>
+      <c r="B140" t="s">
+        <v>233</v>
+      </c>
+      <c r="C140">
+        <v>1200</v>
+      </c>
+      <c r="D140" t="s">
+        <v>379</v>
+      </c>
+      <c r="F140" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>381</v>
+      </c>
+      <c r="B141" t="s">
+        <v>101</v>
+      </c>
+      <c r="C141">
+        <v>1700</v>
+      </c>
+      <c r="D141" t="s">
+        <v>382</v>
+      </c>
+      <c r="F141" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>384</v>
+      </c>
+      <c r="B142" t="s">
+        <v>233</v>
+      </c>
+      <c r="C142">
+        <v>4000</v>
+      </c>
+      <c r="D142" t="s">
+        <v>385</v>
+      </c>
+      <c r="F142" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>387</v>
+      </c>
+      <c r="B143" t="s">
+        <v>158</v>
+      </c>
+      <c r="C143">
+        <v>1000</v>
+      </c>
+      <c r="D143" t="s">
+        <v>388</v>
+      </c>
+      <c r="F143" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>390</v>
+      </c>
+      <c r="B144" t="s">
+        <v>233</v>
+      </c>
+      <c r="C144">
+        <v>1200</v>
+      </c>
+      <c r="D144" t="s">
+        <v>391</v>
+      </c>
+      <c r="F144" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>393</v>
+      </c>
+      <c r="B145" t="s">
+        <v>158</v>
+      </c>
+      <c r="C145">
+        <v>1000</v>
+      </c>
+      <c r="D145" t="s">
+        <v>394</v>
+      </c>
+      <c r="F145" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>396</v>
+      </c>
+      <c r="B146" t="s">
+        <v>158</v>
+      </c>
+      <c r="C146">
+        <v>350</v>
+      </c>
+      <c r="F146" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>398</v>
+      </c>
+      <c r="B147" t="s">
+        <v>158</v>
+      </c>
+      <c r="C147">
+        <v>400</v>
+      </c>
+      <c r="F147" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>400</v>
+      </c>
+      <c r="B148" t="s">
+        <v>101</v>
+      </c>
+      <c r="C148">
+        <v>900</v>
+      </c>
+      <c r="F148" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>402</v>
+      </c>
+      <c r="B149" t="s">
+        <v>101</v>
+      </c>
+      <c r="C149">
+        <v>950</v>
+      </c>
+      <c r="D149" t="s">
+        <v>404</v>
+      </c>
+      <c r="F149" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>405</v>
+      </c>
+      <c r="B150" t="s">
+        <v>101</v>
+      </c>
+      <c r="C150">
+        <v>500</v>
+      </c>
+      <c r="F150" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>407</v>
+      </c>
+      <c r="B151" t="s">
+        <v>101</v>
+      </c>
+      <c r="C151">
+        <v>1050</v>
+      </c>
+      <c r="D151" t="s">
+        <v>408</v>
+      </c>
+      <c r="F151" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>410</v>
+      </c>
+      <c r="B152" t="s">
+        <v>573</v>
+      </c>
+      <c r="C152">
+        <v>1000</v>
+      </c>
+      <c r="F152" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>412</v>
+      </c>
+      <c r="B153" t="s">
+        <v>60</v>
+      </c>
+      <c r="C153">
+        <v>250</v>
+      </c>
+      <c r="D153" t="s">
+        <v>413</v>
+      </c>
+      <c r="F153" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>416</v>
+      </c>
+      <c r="B154" t="s">
+        <v>60</v>
+      </c>
+      <c r="C154">
+        <v>1000</v>
+      </c>
+      <c r="F154" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>417</v>
+      </c>
+      <c r="B155" t="s">
+        <v>233</v>
+      </c>
+      <c r="C155">
+        <v>2000</v>
+      </c>
+      <c r="D155" t="s">
+        <v>418</v>
+      </c>
+      <c r="F155" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>422</v>
+      </c>
+      <c r="B156" t="s">
+        <v>60</v>
+      </c>
+      <c r="C156">
+        <v>350</v>
+      </c>
+      <c r="D156" t="s">
+        <v>420</v>
+      </c>
+      <c r="F156" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>423</v>
+      </c>
+      <c r="B157" t="s">
+        <v>10</v>
+      </c>
+      <c r="C157">
+        <v>1200</v>
+      </c>
+      <c r="D157" t="s">
+        <v>424</v>
+      </c>
+      <c r="F157" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>426</v>
+      </c>
+      <c r="B158" t="s">
+        <v>101</v>
+      </c>
+      <c r="C158">
+        <v>2000</v>
+      </c>
+      <c r="D158" t="s">
+        <v>427</v>
+      </c>
+      <c r="F158" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>429</v>
+      </c>
+      <c r="B159" t="s">
+        <v>101</v>
+      </c>
+      <c r="C159">
+        <v>1500</v>
+      </c>
+      <c r="D159" t="s">
+        <v>430</v>
+      </c>
+      <c r="F159" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>432</v>
+      </c>
+      <c r="B160" t="s">
+        <v>158</v>
+      </c>
+      <c r="C160">
+        <v>400</v>
+      </c>
+      <c r="F160" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>434</v>
+      </c>
+      <c r="B161" t="s">
+        <v>64</v>
+      </c>
+      <c r="C161">
+        <v>2500</v>
+      </c>
+      <c r="D161" t="s">
+        <v>435</v>
+      </c>
+      <c r="F161" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>437</v>
+      </c>
+      <c r="B162" t="s">
+        <v>64</v>
+      </c>
+      <c r="C162">
+        <v>800</v>
+      </c>
+      <c r="D162" t="s">
+        <v>438</v>
+      </c>
+      <c r="F162" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>440</v>
+      </c>
+      <c r="B163" t="s">
+        <v>221</v>
+      </c>
+      <c r="C163">
+        <v>150</v>
+      </c>
+      <c r="D163" t="s">
+        <v>441</v>
+      </c>
+      <c r="F163" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>443</v>
+      </c>
+      <c r="B164" t="s">
+        <v>64</v>
+      </c>
+      <c r="C164">
+        <v>800</v>
+      </c>
+      <c r="D164" t="s">
+        <v>444</v>
+      </c>
+      <c r="F164" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>446</v>
+      </c>
+      <c r="B165" t="s">
+        <v>93</v>
+      </c>
+      <c r="C165">
+        <v>600</v>
+      </c>
+      <c r="D165" t="s">
+        <v>447</v>
+      </c>
+      <c r="F165" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>449</v>
+      </c>
+      <c r="B166" t="s">
+        <v>60</v>
+      </c>
+      <c r="C166">
+        <v>1500</v>
+      </c>
+      <c r="D166" t="s">
+        <v>450</v>
+      </c>
+      <c r="F166" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>452</v>
+      </c>
+      <c r="B167" t="s">
+        <v>64</v>
+      </c>
+      <c r="C167">
+        <v>2500</v>
+      </c>
+      <c r="D167" t="s">
+        <v>453</v>
+      </c>
+      <c r="F167" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>455</v>
+      </c>
+      <c r="B168" t="s">
+        <v>101</v>
+      </c>
+      <c r="C168">
+        <v>3000</v>
+      </c>
+      <c r="F168" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>457</v>
+      </c>
+      <c r="B169" t="s">
+        <v>101</v>
+      </c>
+      <c r="C169">
+        <v>1500</v>
+      </c>
+      <c r="F169" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>459</v>
+      </c>
+      <c r="B170" t="s">
+        <v>101</v>
+      </c>
+      <c r="C170">
+        <v>2000</v>
+      </c>
+      <c r="D170" t="s">
+        <v>460</v>
+      </c>
+      <c r="F170" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>462</v>
+      </c>
+      <c r="B171" t="s">
+        <v>158</v>
+      </c>
+      <c r="C171">
+        <v>1000</v>
+      </c>
+      <c r="F171" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>464</v>
+      </c>
+      <c r="B172" t="s">
+        <v>64</v>
+      </c>
+      <c r="C172">
+        <v>1000</v>
+      </c>
+      <c r="F172" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>467</v>
+      </c>
+      <c r="B173" t="s">
+        <v>101</v>
+      </c>
+      <c r="C173">
+        <v>950</v>
+      </c>
+      <c r="D173" t="s">
+        <v>468</v>
+      </c>
+      <c r="F173" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>469</v>
+      </c>
+      <c r="B174" t="s">
+        <v>101</v>
+      </c>
+      <c r="C174">
+        <v>2200</v>
+      </c>
+      <c r="D174" t="s">
+        <v>470</v>
+      </c>
+      <c r="F174" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>472</v>
+      </c>
+      <c r="B175" t="s">
+        <v>101</v>
+      </c>
+      <c r="C175">
+        <v>1500</v>
+      </c>
+      <c r="D175" t="s">
+        <v>473</v>
+      </c>
+      <c r="F175" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>475</v>
+      </c>
+      <c r="B176" t="s">
+        <v>60</v>
+      </c>
+      <c r="C176">
+        <v>450</v>
+      </c>
+      <c r="D176" t="s">
+        <v>476</v>
+      </c>
+      <c r="F176" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>478</v>
+      </c>
+      <c r="B177" t="s">
+        <v>101</v>
+      </c>
+      <c r="C177">
+        <v>2000</v>
+      </c>
+      <c r="D177" t="s">
+        <v>479</v>
+      </c>
+      <c r="F177" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>481</v>
+      </c>
+      <c r="B178" t="s">
+        <v>60</v>
+      </c>
+      <c r="C178">
+        <v>500</v>
+      </c>
+      <c r="F178" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>483</v>
+      </c>
+      <c r="B179" t="s">
+        <v>101</v>
+      </c>
+      <c r="C179">
+        <v>200</v>
+      </c>
+      <c r="D179" t="s">
+        <v>484</v>
+      </c>
+      <c r="F179" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>486</v>
+      </c>
+      <c r="B180" t="s">
+        <v>60</v>
+      </c>
+      <c r="C180">
+        <v>1500</v>
+      </c>
+      <c r="D180" t="s">
+        <v>487</v>
+      </c>
+      <c r="F180" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>489</v>
+      </c>
+      <c r="B181" t="s">
+        <v>101</v>
+      </c>
+      <c r="C181">
+        <v>1400</v>
+      </c>
+      <c r="D181" t="s">
+        <v>490</v>
+      </c>
+      <c r="F181" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>492</v>
+      </c>
+      <c r="B182" t="s">
+        <v>101</v>
+      </c>
+      <c r="C182">
+        <v>800</v>
+      </c>
+      <c r="D182" t="s">
+        <v>493</v>
+      </c>
+      <c r="F182" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>495</v>
+      </c>
+      <c r="B183" t="s">
+        <v>233</v>
+      </c>
+      <c r="C183">
+        <v>2000</v>
+      </c>
+      <c r="D183" t="s">
+        <v>496</v>
+      </c>
+      <c r="F183" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>498</v>
+      </c>
+      <c r="B184" t="s">
+        <v>573</v>
+      </c>
+      <c r="C184">
+        <v>3500</v>
+      </c>
+      <c r="F184" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>501</v>
+      </c>
+      <c r="B185" t="s">
+        <v>101</v>
+      </c>
+      <c r="C185">
+        <v>1800</v>
+      </c>
+      <c r="D185" t="s">
+        <v>502</v>
+      </c>
+      <c r="F185" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>503</v>
+      </c>
+      <c r="B186" t="s">
+        <v>101</v>
+      </c>
+      <c r="C186">
+        <v>3200</v>
+      </c>
+      <c r="D186" t="s">
+        <v>504</v>
+      </c>
+      <c r="F186" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>506</v>
+      </c>
+      <c r="B187" t="s">
+        <v>101</v>
+      </c>
+      <c r="C187">
+        <v>70</v>
+      </c>
+      <c r="D187" t="s">
+        <v>507</v>
+      </c>
+      <c r="F187" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>509</v>
+      </c>
+      <c r="B188" t="s">
+        <v>101</v>
+      </c>
+      <c r="C188">
+        <v>700</v>
+      </c>
+      <c r="D188" t="s">
+        <v>510</v>
+      </c>
+      <c r="F188" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>512</v>
+      </c>
+      <c r="B189" t="s">
+        <v>60</v>
+      </c>
+      <c r="C189">
+        <v>1500</v>
+      </c>
+      <c r="D189" t="s">
+        <v>513</v>
+      </c>
+      <c r="F189" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>515</v>
+      </c>
+      <c r="B190" t="s">
+        <v>573</v>
+      </c>
+      <c r="C190">
+        <v>500</v>
+      </c>
+      <c r="F190" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>517</v>
+      </c>
+      <c r="B191" t="s">
+        <v>101</v>
+      </c>
+      <c r="C191">
+        <v>2500</v>
+      </c>
+      <c r="F191" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>519</v>
+      </c>
+      <c r="B192" t="s">
+        <v>60</v>
+      </c>
+      <c r="C192">
+        <v>1000</v>
+      </c>
+      <c r="F192" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>522</v>
+      </c>
+      <c r="B193" t="s">
+        <v>573</v>
+      </c>
+      <c r="C193">
+        <v>2000</v>
+      </c>
+      <c r="F193" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>523</v>
+      </c>
+      <c r="B194" t="s">
+        <v>64</v>
+      </c>
+      <c r="C194">
+        <v>800</v>
+      </c>
+      <c r="D194" t="s">
+        <v>524</v>
+      </c>
+      <c r="F194" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>526</v>
+      </c>
+      <c r="B195" t="s">
+        <v>60</v>
+      </c>
+      <c r="C195">
+        <v>1200</v>
+      </c>
+      <c r="F195" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>528</v>
+      </c>
+      <c r="B196" t="s">
+        <v>101</v>
+      </c>
+      <c r="C196">
+        <v>800</v>
+      </c>
+      <c r="D196" t="s">
+        <v>529</v>
+      </c>
+      <c r="F196" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>531</v>
+      </c>
+      <c r="B197" t="s">
+        <v>101</v>
+      </c>
+      <c r="D197" t="s">
+        <v>532</v>
+      </c>
+      <c r="F197" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>533</v>
+      </c>
+      <c r="B198" t="s">
+        <v>10</v>
+      </c>
+      <c r="C198">
+        <v>900</v>
+      </c>
+      <c r="D198" t="s">
+        <v>534</v>
+      </c>
+      <c r="F198" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>536</v>
+      </c>
+      <c r="B199" t="s">
+        <v>101</v>
+      </c>
+      <c r="C199">
+        <v>1000</v>
+      </c>
+      <c r="F199" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>538</v>
+      </c>
+      <c r="B200" t="s">
+        <v>64</v>
+      </c>
+      <c r="C200">
+        <v>400</v>
+      </c>
+      <c r="D200" t="s">
+        <v>539</v>
+      </c>
+      <c r="F200" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>541</v>
+      </c>
+      <c r="B201" t="s">
+        <v>101</v>
+      </c>
+      <c r="C201">
+        <v>200</v>
+      </c>
+      <c r="D201" t="s">
+        <v>542</v>
+      </c>
+      <c r="F201" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>544</v>
+      </c>
+      <c r="B202" t="s">
+        <v>101</v>
+      </c>
+      <c r="C202">
+        <v>300</v>
+      </c>
+      <c r="D202" t="s">
+        <v>545</v>
+      </c>
+      <c r="F202" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>547</v>
+      </c>
+      <c r="B203" t="s">
+        <v>101</v>
+      </c>
+      <c r="C203">
+        <v>2500</v>
+      </c>
+      <c r="D203" t="s">
+        <v>548</v>
+      </c>
+      <c r="F203" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>550</v>
+      </c>
+      <c r="B204" t="s">
+        <v>60</v>
+      </c>
+      <c r="C204">
+        <v>600</v>
+      </c>
+      <c r="D204" t="s">
+        <v>551</v>
+      </c>
+      <c r="F204" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>553</v>
+      </c>
+      <c r="B205" t="s">
+        <v>101</v>
+      </c>
+      <c r="C205">
+        <v>800</v>
+      </c>
+      <c r="D205" t="s">
+        <v>554</v>
+      </c>
+      <c r="F205" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>556</v>
+      </c>
+      <c r="B206" t="s">
+        <v>101</v>
+      </c>
+      <c r="C206">
+        <v>800</v>
+      </c>
+      <c r="D206" t="s">
+        <v>557</v>
+      </c>
+      <c r="F206" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>559</v>
+      </c>
+      <c r="B207" t="s">
+        <v>10</v>
+      </c>
+      <c r="C207">
+        <v>1500</v>
+      </c>
+      <c r="D207" t="s">
+        <v>560</v>
+      </c>
+      <c r="F207" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>562</v>
+      </c>
+      <c r="B208" t="s">
+        <v>101</v>
+      </c>
+      <c r="C208">
+        <v>1700</v>
+      </c>
+      <c r="D208" t="s">
+        <v>563</v>
+      </c>
+      <c r="F208" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>565</v>
+      </c>
+      <c r="B209" t="s">
+        <v>101</v>
+      </c>
+      <c r="C209">
+        <v>70</v>
+      </c>
+      <c r="D209" t="s">
+        <v>566</v>
+      </c>
+      <c r="F209" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>568</v>
+      </c>
+      <c r="B210" t="s">
+        <v>573</v>
+      </c>
+      <c r="C210">
+        <v>1500</v>
+      </c>
+      <c r="F210" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>570</v>
+      </c>
+      <c r="B211" t="s">
+        <v>101</v>
+      </c>
+      <c r="C211">
+        <v>400</v>
+      </c>
+      <c r="D211" t="s">
+        <v>571</v>
+      </c>
+      <c r="F211" t="s">
+        <v>572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new sunflower wristband product
</commit_message>
<xml_diff>
--- a/database_ready-latest.xlsx
+++ b/database_ready-latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allan Muli\Desktop\Nexus Frontend project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1930222E-EEFF-493A-9492-A2530C8F52F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B2BD6-BDB2-4177-AF01-40A564A83DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="579">
   <si>
     <t>Product_Name</t>
   </si>
@@ -1793,6 +1793,18 @@
   </si>
   <si>
     <t>opposites-puzzle.jpg</t>
+  </si>
+  <si>
+    <t>sunflower-wristband.jpg</t>
+  </si>
+  <si>
+    <t>Sunflower wristband</t>
+  </si>
+  <si>
+    <t>35/- per piece or 300 for ten</t>
+  </si>
+  <si>
+    <t>sunflower-insert-card.jpg</t>
   </si>
 </sst>
 </file>
@@ -2636,7 +2648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33272AF2-EBC5-44E6-A157-58E7ECEB284E}">
-  <dimension ref="A1:F211"/>
+  <dimension ref="A1:F212"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" customWidth="1"/>
@@ -2718,7 +2730,7 @@
         <v>269</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>578</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -5986,6 +5998,23 @@
       </c>
       <c r="F211" t="s">
         <v>572</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>576</v>
+      </c>
+      <c r="B212" t="s">
+        <v>10</v>
+      </c>
+      <c r="C212">
+        <v>35</v>
+      </c>
+      <c r="D212" t="s">
+        <v>577</v>
+      </c>
+      <c r="F212" t="s">
+        <v>575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update of product images
</commit_message>
<xml_diff>
--- a/database_ready-latest.xlsx
+++ b/database_ready-latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allan Muli\Desktop\Nexus Frontend project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B2BD6-BDB2-4177-AF01-40A564A83DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0C7FE5C-EED5-42AF-9B80-513479C6E84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{95A1A84D-1CC9-4BCE-B68E-24AE1010798A}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="581">
   <si>
     <t>Product_Name</t>
   </si>
@@ -100,9 +100,6 @@
     <t>180cm*60cm</t>
   </si>
   <si>
-    <t>sensory-tunnel.png</t>
-  </si>
-  <si>
     <t>Busy ADL Board</t>
   </si>
   <si>
@@ -454,9 +451,6 @@
     <t>6ft</t>
   </si>
   <si>
-    <t>trampoline.png</t>
-  </si>
-  <si>
     <t>8ft</t>
   </si>
   <si>
@@ -511,9 +505,6 @@
     <t>hard-stress-ball.png</t>
   </si>
   <si>
-    <t>Beauty Face massager</t>
-  </si>
-  <si>
     <t>Sensory tactile</t>
   </si>
   <si>
@@ -790,9 +781,6 @@
     <t>action-words.jpg</t>
   </si>
   <si>
-    <t>Tactile disc wall</t>
-  </si>
-  <si>
     <t>12" mix colours</t>
   </si>
   <si>
@@ -811,22 +799,10 @@
     <t>mini trampoline</t>
   </si>
   <si>
-    <t>game board</t>
-  </si>
-  <si>
     <t>shape puzzle</t>
   </si>
   <si>
-    <t>mini-trampoline.png</t>
-  </si>
-  <si>
-    <t>game-board.png</t>
-  </si>
-  <si>
     <t>shape-puzzle.png</t>
-  </si>
-  <si>
-    <t>tactile-disc-wall.jpg</t>
   </si>
   <si>
     <t>Plastic ID card with description of invivible disability and emergency contact information</t>
@@ -1805,6 +1781,36 @@
   </si>
   <si>
     <t>sunflower-insert-card.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> face massager - electric</t>
+  </si>
+  <si>
+    <t>Math game</t>
+  </si>
+  <si>
+    <t>math-game.jpg</t>
+  </si>
+  <si>
+    <t>Sensory Tunnel.jpg</t>
+  </si>
+  <si>
+    <t>1meter in size perfect for ambiance in your sensory room or bedroom for soothing  auditory calming input of bubbles, and color changing.</t>
+  </si>
+  <si>
+    <t>trampoline-6ft.jpg</t>
+  </si>
+  <si>
+    <t>trampoline-8ft.jpg</t>
+  </si>
+  <si>
+    <t>trampoline-12ft.jpg</t>
+  </si>
+  <si>
+    <t>trampoline-10ft.jpg</t>
+  </si>
+  <si>
+    <t>mini-trampoline.jpg</t>
   </si>
 </sst>
 </file>
@@ -2648,7 +2654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33272AF2-EBC5-44E6-A157-58E7ECEB284E}">
-  <dimension ref="A1:F212"/>
+  <dimension ref="A1:F209"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" customWidth="1"/>
@@ -2690,7 +2696,7 @@
         <v>1500</v>
       </c>
       <c r="D2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -2710,7 +2716,7 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
@@ -2721,16 +2727,16 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="C4">
         <v>500</v>
       </c>
       <c r="D4" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="F4" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -2752,7 +2758,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
@@ -2761,7 +2767,7 @@
         <v>4500</v>
       </c>
       <c r="D6" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="F6" t="s">
         <v>19</v>
@@ -2778,7 +2784,7 @@
         <v>2500</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="F7" t="s">
         <v>22</v>
@@ -2798,29 +2804,29 @@
         <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>574</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
         <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
       </c>
       <c r="C9">
         <v>3000</v>
       </c>
       <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
         <v>29</v>
-      </c>
-      <c r="F9" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
@@ -2829,540 +2835,540 @@
         <v>4000</v>
       </c>
       <c r="D10" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="F10" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
         <v>31</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
       </c>
       <c r="C11">
         <v>9000</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
         <v>34</v>
-      </c>
-      <c r="B12" t="s">
-        <v>35</v>
       </c>
       <c r="C12">
         <v>3000</v>
       </c>
       <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
         <v>36</v>
-      </c>
-      <c r="F12" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13">
         <v>4000</v>
       </c>
       <c r="D13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F13" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
         <v>40</v>
-      </c>
-      <c r="B14" t="s">
-        <v>41</v>
       </c>
       <c r="C14">
         <v>4000</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s">
         <v>43</v>
-      </c>
-      <c r="B15" t="s">
-        <v>44</v>
       </c>
       <c r="C15">
         <v>12000</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
         <v>46</v>
-      </c>
-      <c r="B16" t="s">
-        <v>47</v>
       </c>
       <c r="C16">
         <v>9500</v>
       </c>
       <c r="D16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" t="s">
         <v>48</v>
-      </c>
-      <c r="F16" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17">
         <v>200</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" t="s">
         <v>52</v>
-      </c>
-      <c r="B18" t="s">
-        <v>53</v>
       </c>
       <c r="C18">
         <v>1000</v>
       </c>
       <c r="F18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
         <v>55</v>
-      </c>
-      <c r="B19" t="s">
-        <v>56</v>
       </c>
       <c r="C19">
         <v>20000</v>
       </c>
       <c r="D19" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" t="s">
         <v>57</v>
-      </c>
-      <c r="F19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="s">
         <v>59</v>
-      </c>
-      <c r="B20" t="s">
-        <v>60</v>
       </c>
       <c r="C20">
         <v>4900</v>
       </c>
       <c r="D20" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" t="s">
         <v>61</v>
-      </c>
-      <c r="F20" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" t="s">
         <v>63</v>
-      </c>
-      <c r="B21" t="s">
-        <v>64</v>
       </c>
       <c r="C21">
         <v>4500</v>
       </c>
       <c r="D21" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="F21" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" t="s">
         <v>63</v>
-      </c>
-      <c r="B22" t="s">
-        <v>64</v>
       </c>
       <c r="C22">
         <v>5000</v>
       </c>
       <c r="D22" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="F22" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" t="s">
         <v>63</v>
-      </c>
-      <c r="B23" t="s">
-        <v>64</v>
       </c>
       <c r="C23">
         <v>3500</v>
       </c>
       <c r="D23" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="F23" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" t="s">
         <v>65</v>
-      </c>
-      <c r="B24" t="s">
-        <v>66</v>
       </c>
       <c r="C24">
         <v>12500</v>
       </c>
       <c r="D24" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="F24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" t="s">
         <v>68</v>
-      </c>
-      <c r="B25" t="s">
-        <v>69</v>
       </c>
       <c r="C25">
         <v>7500</v>
       </c>
       <c r="D25" t="s">
+        <v>69</v>
+      </c>
+      <c r="F25" t="s">
         <v>70</v>
-      </c>
-      <c r="F25" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" t="s">
         <v>72</v>
-      </c>
-      <c r="B26" t="s">
-        <v>73</v>
       </c>
       <c r="C26">
         <v>3500</v>
       </c>
       <c r="D26" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" t="s">
         <v>74</v>
-      </c>
-      <c r="F26" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27">
+        <v>4000</v>
+      </c>
+      <c r="D27" t="s">
         <v>76</v>
       </c>
-      <c r="B27" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27">
-        <v>43799</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
         <v>77</v>
-      </c>
-      <c r="F27" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" t="s">
         <v>79</v>
-      </c>
-      <c r="B28" t="s">
-        <v>80</v>
       </c>
       <c r="C28">
         <v>1200</v>
       </c>
       <c r="F28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="C29">
         <v>2500</v>
       </c>
       <c r="F29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B30" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="C30">
         <v>3000</v>
       </c>
       <c r="F30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B31" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C31">
         <v>3000</v>
       </c>
       <c r="F31" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>86</v>
+      </c>
+      <c r="B32" t="s">
         <v>87</v>
-      </c>
-      <c r="B32" t="s">
-        <v>88</v>
       </c>
       <c r="C32">
         <v>150</v>
       </c>
       <c r="F32" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C33">
         <v>500</v>
       </c>
       <c r="D33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F33" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" t="s">
         <v>92</v>
-      </c>
-      <c r="B34" t="s">
-        <v>93</v>
       </c>
       <c r="C34">
         <v>1000</v>
       </c>
       <c r="F34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C35">
         <v>3500</v>
       </c>
       <c r="D35" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="F35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C36">
         <v>5000</v>
       </c>
       <c r="D36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B37" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="C37">
         <v>2000</v>
       </c>
       <c r="F37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>99</v>
+      </c>
+      <c r="B38" t="s">
         <v>100</v>
-      </c>
-      <c r="B38" t="s">
-        <v>101</v>
       </c>
       <c r="C38">
         <v>3500</v>
       </c>
       <c r="F38" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39">
         <v>2500</v>
       </c>
       <c r="D39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F39" t="s">
         <v>104</v>
-      </c>
-      <c r="F39" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>105</v>
+      </c>
+      <c r="B40" t="s">
         <v>106</v>
-      </c>
-      <c r="B40" t="s">
-        <v>107</v>
       </c>
       <c r="C40">
         <v>4000</v>
       </c>
       <c r="F40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C41">
         <v>10000</v>
       </c>
       <c r="F41" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>110</v>
+      </c>
+      <c r="B42" t="s">
         <v>111</v>
-      </c>
-      <c r="B42" t="s">
-        <v>112</v>
       </c>
       <c r="C42">
         <v>10000</v>
       </c>
       <c r="F42" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C43">
         <v>4000</v>
       </c>
       <c r="D43" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="F43" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C44">
         <v>5000</v>
       </c>
       <c r="D44" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="F44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -3370,13 +3376,13 @@
         <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C45">
         <v>12500</v>
       </c>
       <c r="D45" t="s">
-        <v>16</v>
+        <v>575</v>
       </c>
       <c r="F45" t="s">
         <v>17</v>
@@ -3384,338 +3390,338 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B46" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="C46">
         <v>25000</v>
       </c>
       <c r="F46" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B47" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="C47">
         <v>12000</v>
       </c>
       <c r="F47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>72</v>
+        <v>120</v>
       </c>
       <c r="B48" t="s">
-        <v>279</v>
+        <v>121</v>
       </c>
       <c r="C48">
-        <v>3500</v>
+        <v>4900</v>
       </c>
       <c r="F48" t="s">
-        <v>75</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B49" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C49">
-        <v>4900</v>
+        <v>9000</v>
+      </c>
+      <c r="D49" t="s">
+        <v>125</v>
       </c>
       <c r="F49" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>123</v>
+      </c>
+      <c r="B50" t="s">
         <v>124</v>
       </c>
-      <c r="B50" t="s">
-        <v>125</v>
-      </c>
       <c r="C50">
-        <v>9000</v>
+        <v>11000</v>
       </c>
       <c r="D50" t="s">
+        <v>127</v>
+      </c>
+      <c r="F50" t="s">
         <v>126</v>
-      </c>
-      <c r="F50" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B51" t="s">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="C51">
-        <v>11000</v>
-      </c>
-      <c r="D51" t="s">
-        <v>128</v>
+        <v>9000</v>
       </c>
       <c r="F51" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B52" t="s">
-        <v>66</v>
+        <v>131</v>
       </c>
       <c r="C52">
-        <v>9000</v>
+        <v>3500</v>
       </c>
       <c r="F52" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B53" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C53">
-        <v>3500</v>
+        <v>3000</v>
+      </c>
+      <c r="D53" t="s">
+        <v>287</v>
       </c>
       <c r="F53" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B54" t="s">
-        <v>135</v>
+        <v>65</v>
       </c>
       <c r="C54">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="D54" t="s">
-        <v>295</v>
+        <v>137</v>
       </c>
       <c r="F54" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B55" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C55">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="D55" t="s">
+        <v>96</v>
+      </c>
+      <c r="F55" t="s">
         <v>138</v>
-      </c>
-      <c r="F55" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C56">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="D56" t="s">
-        <v>97</v>
+        <v>139</v>
       </c>
       <c r="F56" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B57" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C57">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="D57" t="s">
         <v>140</v>
       </c>
       <c r="F57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>137</v>
+        <v>303</v>
       </c>
       <c r="B58" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C58">
-        <v>1200</v>
+        <v>8000</v>
       </c>
       <c r="D58" t="s">
-        <v>141</v>
+        <v>305</v>
       </c>
       <c r="F58" t="s">
-        <v>139</v>
+        <v>304</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B59" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C59">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="D59" t="s">
-        <v>313</v>
+        <v>141</v>
       </c>
       <c r="F59" t="s">
-        <v>312</v>
+        <v>254</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>314</v>
+        <v>293</v>
       </c>
       <c r="B60" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C60">
-        <v>15000</v>
+        <v>45000</v>
       </c>
       <c r="D60" t="s">
         <v>142</v>
       </c>
       <c r="F60" t="s">
-        <v>258</v>
+        <v>576</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="B61" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C61">
-        <v>45000</v>
+        <v>55000</v>
       </c>
       <c r="D61" t="s">
         <v>143</v>
       </c>
       <c r="F61" t="s">
-        <v>144</v>
+        <v>577</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="B62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C62">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="D62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F62" t="s">
-        <v>144</v>
+        <v>579</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="B63" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C63">
-        <v>60000</v>
+        <v>68000</v>
       </c>
       <c r="D63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F63" t="s">
-        <v>144</v>
+        <v>578</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>304</v>
+        <v>146</v>
       </c>
       <c r="B64" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="C64">
-        <v>68000</v>
+        <v>4000</v>
       </c>
       <c r="D64" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F64" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B65" t="s">
-        <v>149</v>
+        <v>65</v>
       </c>
       <c r="C65">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="D65" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F65" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B66" t="s">
-        <v>66</v>
+        <v>34</v>
       </c>
       <c r="C66">
-        <v>3500</v>
-      </c>
-      <c r="D66" t="s">
-        <v>153</v>
+        <v>200</v>
       </c>
       <c r="F66" t="s">
         <v>154</v>
@@ -3726,44 +3732,44 @@
         <v>155</v>
       </c>
       <c r="B67" t="s">
-        <v>35</v>
+        <v>156</v>
       </c>
       <c r="C67">
-        <v>200</v>
+        <v>500</v>
+      </c>
+      <c r="D67" t="s">
+        <v>115</v>
       </c>
       <c r="F67" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B68" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C68">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="D68" t="s">
-        <v>116</v>
+        <v>159</v>
       </c>
       <c r="F68" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>160</v>
+        <v>571</v>
       </c>
       <c r="B69" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C69">
-        <v>1000</v>
-      </c>
-      <c r="D69" t="s">
-        <v>161</v>
+        <v>1500</v>
       </c>
       <c r="F69" t="s">
         <v>162</v>
@@ -3777,24 +3783,27 @@
         <v>164</v>
       </c>
       <c r="C70">
-        <v>1500</v>
+        <v>5000</v>
+      </c>
+      <c r="D70" t="s">
+        <v>165</v>
       </c>
       <c r="F70" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B71" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C71">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="D71" t="s">
-        <v>168</v>
+        <v>35</v>
       </c>
       <c r="F71" t="s">
         <v>169</v>
@@ -3805,13 +3814,13 @@
         <v>170</v>
       </c>
       <c r="B72" t="s">
+        <v>65</v>
+      </c>
+      <c r="C72">
+        <v>15000</v>
+      </c>
+      <c r="D72" t="s">
         <v>171</v>
-      </c>
-      <c r="C72">
-        <v>6000</v>
-      </c>
-      <c r="D72" t="s">
-        <v>36</v>
       </c>
       <c r="F72" t="s">
         <v>172</v>
@@ -3819,36 +3828,33 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
+        <v>282</v>
+      </c>
+      <c r="B73" t="s">
         <v>173</v>
       </c>
-      <c r="B73" t="s">
-        <v>66</v>
-      </c>
       <c r="C73">
-        <v>15000</v>
+        <v>7500</v>
       </c>
       <c r="D73" t="s">
-        <v>174</v>
+        <v>281</v>
       </c>
       <c r="F73" t="s">
-        <v>175</v>
+        <v>283</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>290</v>
+        <v>175</v>
       </c>
       <c r="B74" t="s">
         <v>176</v>
       </c>
       <c r="C74">
-        <v>7500</v>
-      </c>
-      <c r="D74" t="s">
-        <v>289</v>
+        <v>6000</v>
       </c>
       <c r="F74" t="s">
-        <v>291</v>
+        <v>177</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
@@ -3856,10 +3862,13 @@
         <v>178</v>
       </c>
       <c r="B75" t="s">
+        <v>173</v>
+      </c>
+      <c r="C75">
+        <v>45000</v>
+      </c>
+      <c r="D75" t="s">
         <v>179</v>
-      </c>
-      <c r="C75">
-        <v>6000</v>
       </c>
       <c r="F75" t="s">
         <v>180</v>
@@ -3867,103 +3876,100 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>103</v>
+        <v>181</v>
       </c>
       <c r="B76" t="s">
-        <v>158</v>
+        <v>43</v>
       </c>
       <c r="C76">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="D76" t="s">
-        <v>104</v>
+        <v>182</v>
       </c>
       <c r="F76" t="s">
-        <v>105</v>
+        <v>183</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B77" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="C77">
-        <v>45000</v>
-      </c>
-      <c r="D77" t="s">
-        <v>182</v>
+        <v>25000</v>
       </c>
       <c r="F77" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B78" t="s">
-        <v>44</v>
-      </c>
-      <c r="C78">
-        <v>10000</v>
+        <v>185</v>
       </c>
       <c r="D78" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F78" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B79" t="s">
-        <v>188</v>
-      </c>
-      <c r="C79">
-        <v>25000</v>
+        <v>10</v>
       </c>
       <c r="F79" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B80" t="s">
-        <v>188</v>
-      </c>
-      <c r="D80" t="s">
-        <v>191</v>
+        <v>10</v>
+      </c>
+      <c r="C80">
+        <v>15000</v>
       </c>
       <c r="F80" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B81" t="s">
         <v>10</v>
       </c>
+      <c r="C81">
+        <v>2500</v>
+      </c>
       <c r="F81" t="s">
-        <v>194</v>
+        <v>265</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
+        <v>194</v>
+      </c>
+      <c r="B82" t="s">
+        <v>65</v>
+      </c>
+      <c r="C82">
+        <v>25000</v>
+      </c>
+      <c r="D82" t="s">
         <v>195</v>
-      </c>
-      <c r="B82" t="s">
-        <v>10</v>
-      </c>
-      <c r="C82">
-        <v>15000</v>
       </c>
       <c r="F82" t="s">
         <v>196</v>
@@ -3971,30 +3977,30 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B83" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="C83">
-        <v>2500</v>
+        <v>12000</v>
       </c>
       <c r="F83" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B84" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="C84">
-        <v>15000</v>
+        <v>500</v>
       </c>
       <c r="D84" t="s">
-        <v>198</v>
+        <v>276</v>
       </c>
       <c r="F84" t="s">
         <v>199</v>
@@ -4002,247 +4008,244 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B85" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="C85">
-        <v>12000</v>
+        <v>300</v>
+      </c>
+      <c r="D85" t="s">
+        <v>275</v>
       </c>
       <c r="F85" t="s">
-        <v>274</v>
+        <v>199</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
+        <v>200</v>
+      </c>
+      <c r="B86" t="s">
+        <v>156</v>
+      </c>
+      <c r="C86">
+        <v>2500</v>
+      </c>
+      <c r="D86" t="s">
+        <v>307</v>
+      </c>
+      <c r="F86" t="s">
         <v>201</v>
-      </c>
-      <c r="B86" t="s">
-        <v>158</v>
-      </c>
-      <c r="C86">
-        <v>500</v>
-      </c>
-      <c r="D86" t="s">
-        <v>284</v>
-      </c>
-      <c r="F86" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B87" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C87">
-        <v>300</v>
+        <v>3000</v>
       </c>
       <c r="D87" t="s">
-        <v>283</v>
+        <v>203</v>
       </c>
       <c r="F87" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B88" t="s">
-        <v>158</v>
+        <v>100</v>
       </c>
       <c r="C88">
-        <v>2500</v>
-      </c>
-      <c r="D88" t="s">
-        <v>315</v>
+        <v>2000</v>
       </c>
       <c r="F88" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B89" t="s">
-        <v>158</v>
+        <v>100</v>
       </c>
       <c r="C89">
-        <v>3000</v>
-      </c>
-      <c r="D89" t="s">
-        <v>206</v>
+        <v>3500</v>
       </c>
       <c r="F89" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B90" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C90">
-        <v>2000</v>
+        <v>2600</v>
       </c>
       <c r="F90" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B91" t="s">
-        <v>101</v>
+        <v>212</v>
       </c>
       <c r="C91">
-        <v>3500</v>
+        <v>500</v>
       </c>
       <c r="F91" t="s">
-        <v>211</v>
+        <v>255</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>212</v>
+        <v>292</v>
       </c>
       <c r="B92" t="s">
-        <v>101</v>
+        <v>214</v>
       </c>
       <c r="C92">
-        <v>2600</v>
+        <v>2800</v>
       </c>
       <c r="F92" t="s">
-        <v>213</v>
+        <v>301</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
+        <v>299</v>
+      </c>
+      <c r="B93" t="s">
         <v>214</v>
       </c>
-      <c r="B93" t="s">
-        <v>215</v>
-      </c>
       <c r="C93">
-        <v>500</v>
+        <v>3000</v>
+      </c>
+      <c r="D93" t="s">
+        <v>298</v>
       </c>
       <c r="F93" t="s">
-        <v>259</v>
+        <v>300</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>300</v>
+        <v>213</v>
       </c>
       <c r="B94" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C94">
-        <v>2800</v>
+        <v>3500</v>
+      </c>
+      <c r="D94" t="s">
+        <v>215</v>
       </c>
       <c r="F94" t="s">
-        <v>309</v>
+        <v>216</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>307</v>
+        <v>217</v>
       </c>
       <c r="B95" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C95">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="D95" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="F95" t="s">
-        <v>308</v>
+        <v>219</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B96" t="s">
-        <v>217</v>
-      </c>
-      <c r="C96">
-        <v>3500</v>
-      </c>
-      <c r="D96" t="s">
         <v>218</v>
       </c>
       <c r="F96" t="s">
-        <v>219</v>
+        <v>267</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B97" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C97">
-        <v>500</v>
-      </c>
-      <c r="D97" t="s">
-        <v>310</v>
+        <v>3000</v>
       </c>
       <c r="F97" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B98" t="s">
-        <v>221</v>
+        <v>272</v>
+      </c>
+      <c r="C98">
+        <v>2800</v>
+      </c>
+      <c r="D98" t="s">
+        <v>225</v>
       </c>
       <c r="F98" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B99" t="s">
-        <v>225</v>
+        <v>164</v>
       </c>
       <c r="C99">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="F99" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B100" t="s">
-        <v>280</v>
+        <v>164</v>
       </c>
       <c r="C100">
-        <v>2800</v>
-      </c>
-      <c r="D100" t="s">
-        <v>228</v>
+        <v>12500</v>
       </c>
       <c r="F100" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
@@ -4250,229 +4253,241 @@
         <v>229</v>
       </c>
       <c r="B101" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
       <c r="C101">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="F101" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B102" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
       <c r="C102">
-        <v>12500</v>
+        <v>500</v>
       </c>
       <c r="F102" t="s">
-        <v>261</v>
+        <v>233</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B103" t="s">
-        <v>233</v>
+        <v>65</v>
       </c>
       <c r="C103">
-        <v>5000</v>
+        <v>8500</v>
+      </c>
+      <c r="D103" t="s">
+        <v>235</v>
       </c>
       <c r="F103" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B104" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C104">
-        <v>500</v>
+        <v>1500</v>
+      </c>
+      <c r="D104" t="s">
+        <v>279</v>
       </c>
       <c r="F104" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B105" t="s">
-        <v>66</v>
+        <v>240</v>
       </c>
       <c r="C105">
-        <v>8500</v>
-      </c>
-      <c r="D105" t="s">
-        <v>238</v>
+        <v>2200</v>
       </c>
       <c r="F105" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="B106" t="s">
-        <v>233</v>
+        <v>65</v>
       </c>
       <c r="C106">
-        <v>1500</v>
+        <v>8500</v>
       </c>
       <c r="D106" t="s">
-        <v>287</v>
+        <v>242</v>
       </c>
       <c r="F106" t="s">
-        <v>241</v>
+        <v>580</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>242</v>
+        <v>572</v>
       </c>
       <c r="B107" t="s">
-        <v>243</v>
+        <v>100</v>
       </c>
       <c r="C107">
-        <v>2200</v>
+        <v>2500</v>
       </c>
       <c r="F107" t="s">
-        <v>244</v>
+        <v>573</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B108" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C108">
-        <v>8500</v>
-      </c>
-      <c r="D108" t="s">
-        <v>245</v>
+        <v>1500</v>
       </c>
       <c r="F108" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="B109" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C109">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F109" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="B110" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C110">
         <v>1500</v>
       </c>
       <c r="F110" t="s">
-        <v>267</v>
+        <v>246</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B111" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C111">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="F111" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B112" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C112">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="F112" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B113" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C113">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="F113" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>252</v>
+        <v>311</v>
       </c>
       <c r="B114" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C114">
-        <v>3000</v>
+        <v>1600</v>
+      </c>
+      <c r="E114" t="s">
+        <v>313</v>
       </c>
       <c r="F114" t="s">
-        <v>253</v>
+        <v>312</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>254</v>
+        <v>314</v>
       </c>
       <c r="B115" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C115">
         <v>3000</v>
       </c>
+      <c r="D115" t="s">
+        <v>316</v>
+      </c>
       <c r="F115" t="s">
-        <v>255</v>
+        <v>315</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>256</v>
+        <v>317</v>
       </c>
       <c r="B116" t="s">
-        <v>101</v>
+        <v>565</v>
+      </c>
+      <c r="C116">
+        <v>2000</v>
+      </c>
+      <c r="D116" t="s">
+        <v>317</v>
       </c>
       <c r="F116" t="s">
-        <v>268</v>
+        <v>318</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
@@ -4480,16 +4495,16 @@
         <v>319</v>
       </c>
       <c r="B117" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C117">
-        <v>1600</v>
-      </c>
-      <c r="E117" t="s">
+        <v>2000</v>
+      </c>
+      <c r="D117" t="s">
+        <v>320</v>
+      </c>
+      <c r="F117" t="s">
         <v>321</v>
-      </c>
-      <c r="F117" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
@@ -4497,16 +4512,16 @@
         <v>322</v>
       </c>
       <c r="B118" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="C118">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="D118" t="s">
+        <v>323</v>
+      </c>
+      <c r="F118" t="s">
         <v>324</v>
-      </c>
-      <c r="F118" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
@@ -4514,30 +4529,27 @@
         <v>325</v>
       </c>
       <c r="B119" t="s">
-        <v>573</v>
+        <v>100</v>
       </c>
       <c r="C119">
-        <v>2000</v>
+        <v>1100</v>
       </c>
       <c r="D119" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F119" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B120" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C120">
-        <v>2000</v>
-      </c>
-      <c r="D120" t="s">
-        <v>328</v>
+        <v>500</v>
       </c>
       <c r="F120" t="s">
         <v>329</v>
@@ -4548,10 +4560,10 @@
         <v>330</v>
       </c>
       <c r="B121" t="s">
-        <v>158</v>
+        <v>100</v>
       </c>
       <c r="C121">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D121" t="s">
         <v>331</v>
@@ -4565,10 +4577,10 @@
         <v>333</v>
       </c>
       <c r="B122" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C122">
-        <v>1100</v>
+        <v>2000</v>
       </c>
       <c r="D122" t="s">
         <v>334</v>
@@ -4582,10 +4594,10 @@
         <v>336</v>
       </c>
       <c r="B123" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C123">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="F123" t="s">
         <v>337</v>
@@ -4593,19 +4605,19 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
+        <v>339</v>
+      </c>
+      <c r="B124" t="s">
+        <v>156</v>
+      </c>
+      <c r="C124">
+        <v>200</v>
+      </c>
+      <c r="D124" t="s">
+        <v>340</v>
+      </c>
+      <c r="F124" t="s">
         <v>338</v>
-      </c>
-      <c r="B124" t="s">
-        <v>101</v>
-      </c>
-      <c r="C124">
-        <v>1500</v>
-      </c>
-      <c r="D124" t="s">
-        <v>339</v>
-      </c>
-      <c r="F124" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
@@ -4613,7 +4625,7 @@
         <v>341</v>
       </c>
       <c r="B125" t="s">
-        <v>101</v>
+        <v>218</v>
       </c>
       <c r="C125">
         <v>2000</v>
@@ -4627,117 +4639,117 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
+        <v>345</v>
+      </c>
+      <c r="B126" t="s">
+        <v>565</v>
+      </c>
+      <c r="C126">
+        <v>1000</v>
+      </c>
+      <c r="F126" t="s">
         <v>344</v>
-      </c>
-      <c r="B126" t="s">
-        <v>101</v>
-      </c>
-      <c r="C126">
-        <v>2000</v>
-      </c>
-      <c r="F126" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
+        <v>346</v>
+      </c>
+      <c r="B127" t="s">
+        <v>230</v>
+      </c>
+      <c r="C127">
+        <v>2300</v>
+      </c>
+      <c r="F127" t="s">
         <v>347</v>
-      </c>
-      <c r="B127" t="s">
-        <v>158</v>
-      </c>
-      <c r="C127">
-        <v>200</v>
-      </c>
-      <c r="D127" t="s">
-        <v>348</v>
-      </c>
-      <c r="F127" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
+        <v>348</v>
+      </c>
+      <c r="B128" t="s">
+        <v>230</v>
+      </c>
+      <c r="C128">
+        <v>1200</v>
+      </c>
+      <c r="F128" t="s">
         <v>349</v>
-      </c>
-      <c r="B128" t="s">
-        <v>221</v>
-      </c>
-      <c r="C128">
-        <v>2000</v>
-      </c>
-      <c r="D128" t="s">
-        <v>350</v>
-      </c>
-      <c r="F128" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B129" t="s">
-        <v>573</v>
+        <v>273</v>
       </c>
       <c r="C129">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="F129" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B130" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C130">
-        <v>2300</v>
+        <v>1600</v>
       </c>
       <c r="F130" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
+        <v>354</v>
+      </c>
+      <c r="B131" t="s">
+        <v>43</v>
+      </c>
+      <c r="C131">
+        <v>250</v>
+      </c>
+      <c r="D131" t="s">
+        <v>355</v>
+      </c>
+      <c r="F131" t="s">
         <v>356</v>
-      </c>
-      <c r="B131" t="s">
-        <v>233</v>
-      </c>
-      <c r="C131">
-        <v>1200</v>
-      </c>
-      <c r="F131" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
+        <v>357</v>
+      </c>
+      <c r="B132" t="s">
+        <v>10</v>
+      </c>
+      <c r="C132">
+        <v>1500</v>
+      </c>
+      <c r="F132" t="s">
         <v>358</v>
-      </c>
-      <c r="B132" t="s">
-        <v>281</v>
-      </c>
-      <c r="C132">
-        <v>600</v>
-      </c>
-      <c r="F132" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
+        <v>359</v>
+      </c>
+      <c r="B133" t="s">
+        <v>100</v>
+      </c>
+      <c r="C133">
+        <v>110</v>
+      </c>
+      <c r="D133" t="s">
         <v>360</v>
-      </c>
-      <c r="B133" t="s">
-        <v>233</v>
-      </c>
-      <c r="C133">
-        <v>1600</v>
       </c>
       <c r="F133" t="s">
         <v>361</v>
@@ -4748,10 +4760,10 @@
         <v>362</v>
       </c>
       <c r="B134" t="s">
-        <v>44</v>
+        <v>230</v>
       </c>
       <c r="C134">
-        <v>250</v>
+        <v>1500</v>
       </c>
       <c r="D134" t="s">
         <v>363</v>
@@ -4765,30 +4777,30 @@
         <v>365</v>
       </c>
       <c r="B135" t="s">
-        <v>10</v>
+        <v>156</v>
       </c>
       <c r="C135">
-        <v>1500</v>
+        <v>600</v>
+      </c>
+      <c r="D135" t="s">
+        <v>366</v>
       </c>
       <c r="F135" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B136" t="s">
-        <v>101</v>
+        <v>230</v>
       </c>
       <c r="C136">
-        <v>110</v>
-      </c>
-      <c r="D136" t="s">
+        <v>2000</v>
+      </c>
+      <c r="F136" t="s">
         <v>368</v>
-      </c>
-      <c r="F136" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
@@ -4796,10 +4808,10 @@
         <v>370</v>
       </c>
       <c r="B137" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C137">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="D137" t="s">
         <v>371</v>
@@ -4813,10 +4825,10 @@
         <v>373</v>
       </c>
       <c r="B138" t="s">
-        <v>158</v>
+        <v>100</v>
       </c>
       <c r="C138">
-        <v>600</v>
+        <v>1700</v>
       </c>
       <c r="D138" t="s">
         <v>374</v>
@@ -4827,81 +4839,81 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
+        <v>376</v>
+      </c>
+      <c r="B139" t="s">
+        <v>230</v>
+      </c>
+      <c r="C139">
+        <v>4000</v>
+      </c>
+      <c r="D139" t="s">
         <v>377</v>
       </c>
-      <c r="B139" t="s">
-        <v>233</v>
-      </c>
-      <c r="C139">
-        <v>2000</v>
-      </c>
       <c r="F139" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B140" t="s">
-        <v>233</v>
+        <v>156</v>
       </c>
       <c r="C140">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="D140" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F140" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B141" t="s">
-        <v>101</v>
+        <v>230</v>
       </c>
       <c r="C141">
-        <v>1700</v>
+        <v>1200</v>
       </c>
       <c r="D141" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F141" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B142" t="s">
-        <v>233</v>
+        <v>156</v>
       </c>
       <c r="C142">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="D142" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F142" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B143" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C143">
-        <v>1000</v>
-      </c>
-      <c r="D143" t="s">
-        <v>388</v>
+        <v>350</v>
       </c>
       <c r="F143" t="s">
         <v>389</v>
@@ -4912,72 +4924,72 @@
         <v>390</v>
       </c>
       <c r="B144" t="s">
-        <v>233</v>
+        <v>156</v>
       </c>
       <c r="C144">
-        <v>1200</v>
-      </c>
-      <c r="D144" t="s">
+        <v>400</v>
+      </c>
+      <c r="F144" t="s">
         <v>391</v>
-      </c>
-      <c r="F144" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
+        <v>392</v>
+      </c>
+      <c r="B145" t="s">
+        <v>100</v>
+      </c>
+      <c r="C145">
+        <v>900</v>
+      </c>
+      <c r="F145" t="s">
         <v>393</v>
-      </c>
-      <c r="B145" t="s">
-        <v>158</v>
-      </c>
-      <c r="C145">
-        <v>1000</v>
-      </c>
-      <c r="D145" t="s">
-        <v>394</v>
-      </c>
-      <c r="F145" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
+        <v>394</v>
+      </c>
+      <c r="B146" t="s">
+        <v>100</v>
+      </c>
+      <c r="C146">
+        <v>950</v>
+      </c>
+      <c r="D146" t="s">
         <v>396</v>
       </c>
-      <c r="B146" t="s">
-        <v>158</v>
-      </c>
-      <c r="C146">
-        <v>350</v>
-      </c>
       <c r="F146" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
+        <v>397</v>
+      </c>
+      <c r="B147" t="s">
+        <v>100</v>
+      </c>
+      <c r="C147">
+        <v>500</v>
+      </c>
+      <c r="F147" t="s">
         <v>398</v>
-      </c>
-      <c r="B147" t="s">
-        <v>158</v>
-      </c>
-      <c r="C147">
-        <v>400</v>
-      </c>
-      <c r="F147" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
+        <v>399</v>
+      </c>
+      <c r="B148" t="s">
+        <v>100</v>
+      </c>
+      <c r="C148">
+        <v>1050</v>
+      </c>
+      <c r="D148" t="s">
         <v>400</v>
-      </c>
-      <c r="B148" t="s">
-        <v>101</v>
-      </c>
-      <c r="C148">
-        <v>900</v>
       </c>
       <c r="F148" t="s">
         <v>401</v>
@@ -4988,13 +5000,10 @@
         <v>402</v>
       </c>
       <c r="B149" t="s">
-        <v>101</v>
+        <v>565</v>
       </c>
       <c r="C149">
-        <v>950</v>
-      </c>
-      <c r="D149" t="s">
-        <v>404</v>
+        <v>1000</v>
       </c>
       <c r="F149" t="s">
         <v>403</v>
@@ -5002,13 +5011,16 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
+        <v>404</v>
+      </c>
+      <c r="B150" t="s">
+        <v>59</v>
+      </c>
+      <c r="C150">
+        <v>250</v>
+      </c>
+      <c r="D150" t="s">
         <v>405</v>
-      </c>
-      <c r="B150" t="s">
-        <v>101</v>
-      </c>
-      <c r="C150">
-        <v>500</v>
       </c>
       <c r="F150" t="s">
         <v>406</v>
@@ -5016,30 +5028,30 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
+        <v>408</v>
+      </c>
+      <c r="B151" t="s">
+        <v>59</v>
+      </c>
+      <c r="C151">
+        <v>1000</v>
+      </c>
+      <c r="F151" t="s">
         <v>407</v>
-      </c>
-      <c r="B151" t="s">
-        <v>101</v>
-      </c>
-      <c r="C151">
-        <v>1050</v>
-      </c>
-      <c r="D151" t="s">
-        <v>408</v>
-      </c>
-      <c r="F151" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
+        <v>409</v>
+      </c>
+      <c r="B152" t="s">
+        <v>230</v>
+      </c>
+      <c r="C152">
+        <v>2000</v>
+      </c>
+      <c r="D152" t="s">
         <v>410</v>
-      </c>
-      <c r="B152" t="s">
-        <v>573</v>
-      </c>
-      <c r="C152">
-        <v>1000</v>
       </c>
       <c r="F152" t="s">
         <v>411</v>
@@ -5047,81 +5059,81 @@
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
+        <v>414</v>
+      </c>
+      <c r="B153" t="s">
+        <v>59</v>
+      </c>
+      <c r="C153">
+        <v>350</v>
+      </c>
+      <c r="D153" t="s">
         <v>412</v>
       </c>
-      <c r="B153" t="s">
-        <v>60</v>
-      </c>
-      <c r="C153">
-        <v>250</v>
-      </c>
-      <c r="D153" t="s">
+      <c r="F153" t="s">
         <v>413</v>
-      </c>
-      <c r="F153" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
+        <v>415</v>
+      </c>
+      <c r="B154" t="s">
+        <v>10</v>
+      </c>
+      <c r="C154">
+        <v>1200</v>
+      </c>
+      <c r="D154" t="s">
         <v>416</v>
       </c>
-      <c r="B154" t="s">
-        <v>60</v>
-      </c>
-      <c r="C154">
-        <v>1000</v>
-      </c>
       <c r="F154" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B155" t="s">
-        <v>233</v>
+        <v>100</v>
       </c>
       <c r="C155">
         <v>2000</v>
       </c>
       <c r="D155" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F155" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
+        <v>421</v>
+      </c>
+      <c r="B156" t="s">
+        <v>100</v>
+      </c>
+      <c r="C156">
+        <v>1500</v>
+      </c>
+      <c r="D156" t="s">
         <v>422</v>
       </c>
-      <c r="B156" t="s">
-        <v>60</v>
-      </c>
-      <c r="C156">
-        <v>350</v>
-      </c>
-      <c r="D156" t="s">
-        <v>420</v>
-      </c>
       <c r="F156" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B157" t="s">
-        <v>10</v>
+        <v>156</v>
       </c>
       <c r="C157">
-        <v>1200</v>
-      </c>
-      <c r="D157" t="s">
-        <v>424</v>
+        <v>400</v>
       </c>
       <c r="F157" t="s">
         <v>425</v>
@@ -5132,10 +5144,10 @@
         <v>426</v>
       </c>
       <c r="B158" t="s">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="C158">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="D158" t="s">
         <v>427</v>
@@ -5149,10 +5161,10 @@
         <v>429</v>
       </c>
       <c r="B159" t="s">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="C159">
-        <v>1500</v>
+        <v>800</v>
       </c>
       <c r="D159" t="s">
         <v>430</v>
@@ -5166,95 +5178,95 @@
         <v>432</v>
       </c>
       <c r="B160" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
       <c r="C160">
-        <v>400</v>
+        <v>150</v>
+      </c>
+      <c r="D160" t="s">
+        <v>433</v>
       </c>
       <c r="F160" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B161" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C161">
-        <v>2500</v>
+        <v>800</v>
       </c>
       <c r="D161" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F161" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B162" t="s">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="C162">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="D162" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F162" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B163" t="s">
-        <v>221</v>
+        <v>59</v>
       </c>
       <c r="C163">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="D163" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F163" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B164" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C164">
-        <v>800</v>
+        <v>2500</v>
       </c>
       <c r="D164" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F164" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B165" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C165">
-        <v>600</v>
-      </c>
-      <c r="D165" t="s">
-        <v>447</v>
+        <v>3000</v>
       </c>
       <c r="F165" t="s">
         <v>448</v>
@@ -5265,61 +5277,58 @@
         <v>449</v>
       </c>
       <c r="B166" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C166">
         <v>1500</v>
       </c>
-      <c r="D166" t="s">
+      <c r="F166" t="s">
         <v>450</v>
-      </c>
-      <c r="F166" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
+        <v>451</v>
+      </c>
+      <c r="B167" t="s">
+        <v>100</v>
+      </c>
+      <c r="C167">
+        <v>2000</v>
+      </c>
+      <c r="D167" t="s">
         <v>452</v>
       </c>
-      <c r="B167" t="s">
-        <v>64</v>
-      </c>
-      <c r="C167">
-        <v>2500</v>
-      </c>
-      <c r="D167" t="s">
+      <c r="F167" t="s">
         <v>453</v>
-      </c>
-      <c r="F167" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
+        <v>454</v>
+      </c>
+      <c r="B168" t="s">
+        <v>156</v>
+      </c>
+      <c r="C168">
+        <v>1000</v>
+      </c>
+      <c r="F168" t="s">
         <v>455</v>
-      </c>
-      <c r="B168" t="s">
-        <v>101</v>
-      </c>
-      <c r="C168">
-        <v>3000</v>
-      </c>
-      <c r="F168" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
+        <v>456</v>
+      </c>
+      <c r="B169" t="s">
+        <v>63</v>
+      </c>
+      <c r="C169">
+        <v>1000</v>
+      </c>
+      <c r="F169" t="s">
         <v>457</v>
-      </c>
-      <c r="B169" t="s">
-        <v>101</v>
-      </c>
-      <c r="C169">
-        <v>1500</v>
-      </c>
-      <c r="F169" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
@@ -5327,27 +5336,30 @@
         <v>459</v>
       </c>
       <c r="B170" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C170">
-        <v>2000</v>
+        <v>950</v>
       </c>
       <c r="D170" t="s">
         <v>460</v>
       </c>
       <c r="F170" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
+        <v>461</v>
+      </c>
+      <c r="B171" t="s">
+        <v>100</v>
+      </c>
+      <c r="C171">
+        <v>2200</v>
+      </c>
+      <c r="D171" t="s">
         <v>462</v>
-      </c>
-      <c r="B171" t="s">
-        <v>158</v>
-      </c>
-      <c r="C171">
-        <v>1000</v>
       </c>
       <c r="F171" t="s">
         <v>463</v>
@@ -5358,13 +5370,16 @@
         <v>464</v>
       </c>
       <c r="B172" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="C172">
-        <v>1000</v>
+        <v>1500</v>
+      </c>
+      <c r="D172" t="s">
+        <v>465</v>
       </c>
       <c r="F172" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
@@ -5372,47 +5387,44 @@
         <v>467</v>
       </c>
       <c r="B173" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C173">
-        <v>950</v>
+        <v>450</v>
       </c>
       <c r="D173" t="s">
         <v>468</v>
       </c>
       <c r="F173" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B174" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C174">
-        <v>2200</v>
+        <v>2000</v>
       </c>
       <c r="D174" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F174" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B175" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C175">
-        <v>1500</v>
-      </c>
-      <c r="D175" t="s">
-        <v>473</v>
+        <v>500</v>
       </c>
       <c r="F175" t="s">
         <v>474</v>
@@ -5423,10 +5435,10 @@
         <v>475</v>
       </c>
       <c r="B176" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C176">
-        <v>450</v>
+        <v>200</v>
       </c>
       <c r="D176" t="s">
         <v>476</v>
@@ -5440,10 +5452,10 @@
         <v>478</v>
       </c>
       <c r="B177" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C177">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D177" t="s">
         <v>479</v>
@@ -5457,61 +5469,61 @@
         <v>481</v>
       </c>
       <c r="B178" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C178">
-        <v>500</v>
+        <v>1400</v>
+      </c>
+      <c r="D178" t="s">
+        <v>482</v>
       </c>
       <c r="F178" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B179" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C179">
-        <v>200</v>
+        <v>800</v>
       </c>
       <c r="D179" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F179" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B180" t="s">
-        <v>60</v>
+        <v>230</v>
       </c>
       <c r="C180">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="D180" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F180" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B181" t="s">
-        <v>101</v>
+        <v>565</v>
       </c>
       <c r="C181">
-        <v>1400</v>
-      </c>
-      <c r="D181" t="s">
-        <v>490</v>
+        <v>3500</v>
       </c>
       <c r="F181" t="s">
         <v>491</v>
@@ -5519,19 +5531,19 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
+        <v>493</v>
+      </c>
+      <c r="B182" t="s">
+        <v>100</v>
+      </c>
+      <c r="C182">
+        <v>1800</v>
+      </c>
+      <c r="D182" t="s">
+        <v>494</v>
+      </c>
+      <c r="F182" t="s">
         <v>492</v>
-      </c>
-      <c r="B182" t="s">
-        <v>101</v>
-      </c>
-      <c r="C182">
-        <v>800</v>
-      </c>
-      <c r="D182" t="s">
-        <v>493</v>
-      </c>
-      <c r="F182" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
@@ -5539,10 +5551,10 @@
         <v>495</v>
       </c>
       <c r="B183" t="s">
-        <v>233</v>
+        <v>100</v>
       </c>
       <c r="C183">
-        <v>2000</v>
+        <v>3200</v>
       </c>
       <c r="D183" t="s">
         <v>496</v>
@@ -5556,13 +5568,16 @@
         <v>498</v>
       </c>
       <c r="B184" t="s">
-        <v>573</v>
+        <v>100</v>
       </c>
       <c r="C184">
-        <v>3500</v>
+        <v>70</v>
+      </c>
+      <c r="D184" t="s">
+        <v>499</v>
       </c>
       <c r="F184" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
@@ -5570,47 +5585,44 @@
         <v>501</v>
       </c>
       <c r="B185" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C185">
-        <v>1800</v>
+        <v>700</v>
       </c>
       <c r="D185" t="s">
         <v>502</v>
       </c>
       <c r="F185" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B186" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C186">
-        <v>3200</v>
+        <v>1500</v>
       </c>
       <c r="D186" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F186" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B187" t="s">
-        <v>101</v>
+        <v>565</v>
       </c>
       <c r="C187">
-        <v>70</v>
-      </c>
-      <c r="D187" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="F187" t="s">
         <v>508</v>
@@ -5621,89 +5633,89 @@
         <v>509</v>
       </c>
       <c r="B188" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C188">
-        <v>700</v>
-      </c>
-      <c r="D188" t="s">
+        <v>2500</v>
+      </c>
+      <c r="F188" t="s">
         <v>510</v>
-      </c>
-      <c r="F188" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
+        <v>511</v>
+      </c>
+      <c r="B189" t="s">
+        <v>59</v>
+      </c>
+      <c r="C189">
+        <v>1000</v>
+      </c>
+      <c r="F189" t="s">
         <v>512</v>
-      </c>
-      <c r="B189" t="s">
-        <v>60</v>
-      </c>
-      <c r="C189">
-        <v>1500</v>
-      </c>
-      <c r="D189" t="s">
-        <v>513</v>
-      </c>
-      <c r="F189" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B190" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="C190">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="F190" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
+        <v>515</v>
+      </c>
+      <c r="B191" t="s">
+        <v>63</v>
+      </c>
+      <c r="C191">
+        <v>800</v>
+      </c>
+      <c r="D191" t="s">
+        <v>516</v>
+      </c>
+      <c r="F191" t="s">
         <v>517</v>
-      </c>
-      <c r="B191" t="s">
-        <v>101</v>
-      </c>
-      <c r="C191">
-        <v>2500</v>
-      </c>
-      <c r="F191" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
+        <v>518</v>
+      </c>
+      <c r="B192" t="s">
+        <v>59</v>
+      </c>
+      <c r="C192">
+        <v>1200</v>
+      </c>
+      <c r="F192" t="s">
         <v>519</v>
-      </c>
-      <c r="B192" t="s">
-        <v>60</v>
-      </c>
-      <c r="C192">
-        <v>1000</v>
-      </c>
-      <c r="F192" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
+        <v>520</v>
+      </c>
+      <c r="B193" t="s">
+        <v>100</v>
+      </c>
+      <c r="C193">
+        <v>800</v>
+      </c>
+      <c r="D193" t="s">
+        <v>521</v>
+      </c>
+      <c r="F193" t="s">
         <v>522</v>
-      </c>
-      <c r="B193" t="s">
-        <v>573</v>
-      </c>
-      <c r="C193">
-        <v>2000</v>
-      </c>
-      <c r="F193" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
@@ -5711,27 +5723,27 @@
         <v>523</v>
       </c>
       <c r="B194" t="s">
-        <v>64</v>
-      </c>
-      <c r="C194">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="D194" t="s">
         <v>524</v>
       </c>
       <c r="F194" t="s">
-        <v>525</v>
+        <v>566</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
+        <v>525</v>
+      </c>
+      <c r="B195" t="s">
+        <v>10</v>
+      </c>
+      <c r="C195">
+        <v>900</v>
+      </c>
+      <c r="D195" t="s">
         <v>526</v>
-      </c>
-      <c r="B195" t="s">
-        <v>60</v>
-      </c>
-      <c r="C195">
-        <v>1200</v>
       </c>
       <c r="F195" t="s">
         <v>527</v>
@@ -5742,30 +5754,30 @@
         <v>528</v>
       </c>
       <c r="B196" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C196">
-        <v>800</v>
-      </c>
-      <c r="D196" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F196" t="s">
         <v>529</v>
-      </c>
-      <c r="F196" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
+        <v>530</v>
+      </c>
+      <c r="B197" t="s">
+        <v>63</v>
+      </c>
+      <c r="C197">
+        <v>400</v>
+      </c>
+      <c r="D197" t="s">
         <v>531</v>
       </c>
-      <c r="B197" t="s">
-        <v>101</v>
-      </c>
-      <c r="D197" t="s">
+      <c r="F197" t="s">
         <v>532</v>
-      </c>
-      <c r="F197" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
@@ -5773,10 +5785,10 @@
         <v>533</v>
       </c>
       <c r="B198" t="s">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="C198">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="D198" t="s">
         <v>534</v>
@@ -5790,146 +5802,146 @@
         <v>536</v>
       </c>
       <c r="B199" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C199">
-        <v>1000</v>
+        <v>300</v>
+      </c>
+      <c r="D199" t="s">
+        <v>537</v>
       </c>
       <c r="F199" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B200" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="C200">
-        <v>400</v>
+        <v>2500</v>
       </c>
       <c r="D200" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F200" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B201" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C201">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="D201" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F201" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B202" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C202">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="D202" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="F202" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B203" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C203">
-        <v>2500</v>
+        <v>800</v>
       </c>
       <c r="D203" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="F203" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B204" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C204">
-        <v>600</v>
+        <v>1500</v>
       </c>
       <c r="D204" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F204" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B205" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C205">
-        <v>800</v>
+        <v>1700</v>
       </c>
       <c r="D205" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="F205" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B206" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C206">
-        <v>800</v>
+        <v>70</v>
       </c>
       <c r="D206" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F206" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B207" t="s">
-        <v>10</v>
+        <v>565</v>
       </c>
       <c r="C207">
         <v>1500</v>
-      </c>
-      <c r="D207" t="s">
-        <v>560</v>
       </c>
       <c r="F207" t="s">
         <v>561</v>
@@ -5940,10 +5952,10 @@
         <v>562</v>
       </c>
       <c r="B208" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C208">
-        <v>1700</v>
+        <v>400</v>
       </c>
       <c r="D208" t="s">
         <v>563</v>
@@ -5954,67 +5966,19 @@
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B209" t="s">
-        <v>101</v>
+        <v>10</v>
       </c>
       <c r="C209">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="D209" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="F209" t="s">
         <v>567</v>
-      </c>
-    </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A210" t="s">
-        <v>568</v>
-      </c>
-      <c r="B210" t="s">
-        <v>573</v>
-      </c>
-      <c r="C210">
-        <v>1500</v>
-      </c>
-      <c r="F210" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A211" t="s">
-        <v>570</v>
-      </c>
-      <c r="B211" t="s">
-        <v>101</v>
-      </c>
-      <c r="C211">
-        <v>400</v>
-      </c>
-      <c r="D211" t="s">
-        <v>571</v>
-      </c>
-      <c r="F211" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A212" t="s">
-        <v>576</v>
-      </c>
-      <c r="B212" t="s">
-        <v>10</v>
-      </c>
-      <c r="C212">
-        <v>35</v>
-      </c>
-      <c r="D212" t="s">
-        <v>577</v>
-      </c>
-      <c r="F212" t="s">
-        <v>575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>